<commit_message>
Regenerate example results without hand-glued keys
</commit_message>
<xml_diff>
--- a/ejemplos/resultados/departamento.xlsx
+++ b/ejemplos/resultados/departamento.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="Asignacion">OFFSET('Asignacion'!$A$4,0,0,COUNTA('Asignacion'!$A$4:$A$34),12)</definedName>
+    <definedName name="Asignacion">OFFSET('Asignacion'!$A$4,0,0,COUNTA('Asignacion'!$A$4:$A$34),11)</definedName>
     <definedName name="Profesores">OFFSET('Carga por profesor'!$A$4,0,0,COUNTA('Carga por profesor'!$A$4:$A$27),7)</definedName>
     <definedName name="Asignaturas">OFFSET('Cobertura por asignatura'!$A$4,0,0,COUNTA('Cobertura por asignatura'!$A$4:$A$27),12)</definedName>
   </definedNames>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -516,12 +516,11 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col hidden="1" width="24" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,30 +573,25 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Par</t>
+          <t>Codigo</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Codigo</t>
+          <t>Primera del par</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Primera del par</t>
+          <t>Cuenta</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Cuenta</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>(nivel de las marcas)</t>
         </is>
@@ -636,26 +630,22 @@
         <v/>
       </c>
       <c r="I4" s="3">
-        <f>IF(AND($A4=""),"",IF(OR(($E4=""),($B4="")),"",(IF(ISNUMBER($E4),IF($E4=0,"0",ROUND($E4,9-INT(LOG10(ABS($E4))))&amp;""),$E4&amp;"")&amp;"|"&amp;IF(ISNUMBER($B4),IF($B4=0,"0",ROUND($B4,9-INT(LOG10(ABS($B4))))&amp;""),$B4&amp;""))))</f>
+        <f>IF(AND($A4=""),"",(IF(ISNUMBER($B4),IF($B4=0,"0",ROUND($B4,9-INT(LOG10(ABS($B4))))&amp;""),$B4&amp;"")&amp;" "&amp;IF(ISNUMBER($C4),IF($C4=0,"0",ROUND($C4,9-INT(LOG10(ABS($C4))))&amp;""),$C4&amp;"")&amp;" "&amp;IF(ISNUMBER($D4),IF($D4=0,"0",ROUND($D4,9-INT(LOG10(ABS($D4))))&amp;""),$D4&amp;"")))</f>
         <v/>
       </c>
       <c r="J4" s="3">
-        <f>IF(AND($A4=""),"",(IF(ISNUMBER($B4),IF($B4=0,"0",ROUND($B4,9-INT(LOG10(ABS($B4))))&amp;""),$B4&amp;"")&amp;" "&amp;IF(ISNUMBER($C4),IF($C4=0,"0",ROUND($C4,9-INT(LOG10(ABS($C4))))&amp;""),$C4&amp;"")&amp;" "&amp;IF(ISNUMBER($D4),IF($D4=0,"0",ROUND($D4,9-INT(LOG10(ABS($D4))))&amp;""),$D4&amp;"")))</f>
+        <f>IF(AND($A4=""),"",IF(OR(($E4=""),($B4="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E4))*(EXACT('Asignacion'!$B$4:$B$34,$B4)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E4))*(EXACT('Asignacion'!$B$4:$B$34,$B4)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E4))*(EXACT('Asignacion'!$B$4:$B$34,$B4)),0),0))))))</f>
         <v/>
       </c>
       <c r="K4" s="3">
-        <f>IF(AND($A4=""),"",IF(EXACT($I4,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I4)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I4)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I4)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A4=""),"",IF(AND(NOT(EXACT($J4,"")),EXACT($J4,$I4)),1,0))</f>
         <v/>
       </c>
       <c r="L4" s="3">
-        <f>IF(AND($A4=""),"",IF(AND(NOT(EXACT($I4,"")),EXACT($K4,$J4)),1,0))</f>
+        <f>IF(AND($A4=""),"",MID(IF(AND(NOT(($B4="")),($E4="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M4" s="3">
-        <f>IF(AND($A4=""),"",MID(IF(AND(NOT(($B4="")),($E4="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N4" s="3">
         <f>IF(OR(AND(NOT(($B4="")),($E4=""))),2,0)</f>
         <v/>
       </c>
@@ -697,26 +687,22 @@
         <v/>
       </c>
       <c r="I5" s="3">
-        <f>IF(AND($A5=""),"",IF(OR(($E5=""),($B5="")),"",(IF(ISNUMBER($E5),IF($E5=0,"0",ROUND($E5,9-INT(LOG10(ABS($E5))))&amp;""),$E5&amp;"")&amp;"|"&amp;IF(ISNUMBER($B5),IF($B5=0,"0",ROUND($B5,9-INT(LOG10(ABS($B5))))&amp;""),$B5&amp;""))))</f>
+        <f>IF(AND($A5=""),"",(IF(ISNUMBER($B5),IF($B5=0,"0",ROUND($B5,9-INT(LOG10(ABS($B5))))&amp;""),$B5&amp;"")&amp;" "&amp;IF(ISNUMBER($C5),IF($C5=0,"0",ROUND($C5,9-INT(LOG10(ABS($C5))))&amp;""),$C5&amp;"")&amp;" "&amp;IF(ISNUMBER($D5),IF($D5=0,"0",ROUND($D5,9-INT(LOG10(ABS($D5))))&amp;""),$D5&amp;"")))</f>
         <v/>
       </c>
       <c r="J5" s="3">
-        <f>IF(AND($A5=""),"",(IF(ISNUMBER($B5),IF($B5=0,"0",ROUND($B5,9-INT(LOG10(ABS($B5))))&amp;""),$B5&amp;"")&amp;" "&amp;IF(ISNUMBER($C5),IF($C5=0,"0",ROUND($C5,9-INT(LOG10(ABS($C5))))&amp;""),$C5&amp;"")&amp;" "&amp;IF(ISNUMBER($D5),IF($D5=0,"0",ROUND($D5,9-INT(LOG10(ABS($D5))))&amp;""),$D5&amp;"")))</f>
+        <f>IF(AND($A5=""),"",IF(OR(($E5=""),($B5="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E5))*(EXACT('Asignacion'!$B$4:$B$34,$B5)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E5))*(EXACT('Asignacion'!$B$4:$B$34,$B5)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E5))*(EXACT('Asignacion'!$B$4:$B$34,$B5)),0),0))))))</f>
         <v/>
       </c>
       <c r="K5" s="3">
-        <f>IF(AND($A5=""),"",IF(EXACT($I5,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I5)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I5)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I5)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A5=""),"",IF(AND(NOT(EXACT($J5,"")),EXACT($J5,$I5)),1,0))</f>
         <v/>
       </c>
       <c r="L5" s="3">
-        <f>IF(AND($A5=""),"",IF(AND(NOT(EXACT($I5,"")),EXACT($K5,$J5)),1,0))</f>
+        <f>IF(AND($A5=""),"",MID(IF(AND(NOT(($B5="")),($E5="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M5" s="3">
-        <f>IF(AND($A5=""),"",MID(IF(AND(NOT(($B5="")),($E5="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N5" s="3">
         <f>IF(OR(AND(NOT(($B5="")),($E5=""))),2,0)</f>
         <v/>
       </c>
@@ -758,26 +744,22 @@
         <v/>
       </c>
       <c r="I6" s="3">
-        <f>IF(AND($A6=""),"",IF(OR(($E6=""),($B6="")),"",(IF(ISNUMBER($E6),IF($E6=0,"0",ROUND($E6,9-INT(LOG10(ABS($E6))))&amp;""),$E6&amp;"")&amp;"|"&amp;IF(ISNUMBER($B6),IF($B6=0,"0",ROUND($B6,9-INT(LOG10(ABS($B6))))&amp;""),$B6&amp;""))))</f>
+        <f>IF(AND($A6=""),"",(IF(ISNUMBER($B6),IF($B6=0,"0",ROUND($B6,9-INT(LOG10(ABS($B6))))&amp;""),$B6&amp;"")&amp;" "&amp;IF(ISNUMBER($C6),IF($C6=0,"0",ROUND($C6,9-INT(LOG10(ABS($C6))))&amp;""),$C6&amp;"")&amp;" "&amp;IF(ISNUMBER($D6),IF($D6=0,"0",ROUND($D6,9-INT(LOG10(ABS($D6))))&amp;""),$D6&amp;"")))</f>
         <v/>
       </c>
       <c r="J6" s="3">
-        <f>IF(AND($A6=""),"",(IF(ISNUMBER($B6),IF($B6=0,"0",ROUND($B6,9-INT(LOG10(ABS($B6))))&amp;""),$B6&amp;"")&amp;" "&amp;IF(ISNUMBER($C6),IF($C6=0,"0",ROUND($C6,9-INT(LOG10(ABS($C6))))&amp;""),$C6&amp;"")&amp;" "&amp;IF(ISNUMBER($D6),IF($D6=0,"0",ROUND($D6,9-INT(LOG10(ABS($D6))))&amp;""),$D6&amp;"")))</f>
+        <f>IF(AND($A6=""),"",IF(OR(($E6=""),($B6="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E6))*(EXACT('Asignacion'!$B$4:$B$34,$B6)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E6))*(EXACT('Asignacion'!$B$4:$B$34,$B6)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E6))*(EXACT('Asignacion'!$B$4:$B$34,$B6)),0),0))))))</f>
         <v/>
       </c>
       <c r="K6" s="3">
-        <f>IF(AND($A6=""),"",IF(EXACT($I6,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I6)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I6)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I6)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A6=""),"",IF(AND(NOT(EXACT($J6,"")),EXACT($J6,$I6)),1,0))</f>
         <v/>
       </c>
       <c r="L6" s="3">
-        <f>IF(AND($A6=""),"",IF(AND(NOT(EXACT($I6,"")),EXACT($K6,$J6)),1,0))</f>
+        <f>IF(AND($A6=""),"",MID(IF(AND(NOT(($B6="")),($E6="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M6" s="3">
-        <f>IF(AND($A6=""),"",MID(IF(AND(NOT(($B6="")),($E6="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N6" s="3">
         <f>IF(OR(AND(NOT(($B6="")),($E6=""))),2,0)</f>
         <v/>
       </c>
@@ -815,26 +797,22 @@
         <v/>
       </c>
       <c r="I7" s="3">
-        <f>IF(AND($A7=""),"",IF(OR(($E7=""),($B7="")),"",(IF(ISNUMBER($E7),IF($E7=0,"0",ROUND($E7,9-INT(LOG10(ABS($E7))))&amp;""),$E7&amp;"")&amp;"|"&amp;IF(ISNUMBER($B7),IF($B7=0,"0",ROUND($B7,9-INT(LOG10(ABS($B7))))&amp;""),$B7&amp;""))))</f>
+        <f>IF(AND($A7=""),"",(IF(ISNUMBER($B7),IF($B7=0,"0",ROUND($B7,9-INT(LOG10(ABS($B7))))&amp;""),$B7&amp;"")&amp;" "&amp;IF(ISNUMBER($C7),IF($C7=0,"0",ROUND($C7,9-INT(LOG10(ABS($C7))))&amp;""),$C7&amp;"")&amp;" "&amp;IF(ISNUMBER($D7),IF($D7=0,"0",ROUND($D7,9-INT(LOG10(ABS($D7))))&amp;""),$D7&amp;"")))</f>
         <v/>
       </c>
       <c r="J7" s="3">
-        <f>IF(AND($A7=""),"",(IF(ISNUMBER($B7),IF($B7=0,"0",ROUND($B7,9-INT(LOG10(ABS($B7))))&amp;""),$B7&amp;"")&amp;" "&amp;IF(ISNUMBER($C7),IF($C7=0,"0",ROUND($C7,9-INT(LOG10(ABS($C7))))&amp;""),$C7&amp;"")&amp;" "&amp;IF(ISNUMBER($D7),IF($D7=0,"0",ROUND($D7,9-INT(LOG10(ABS($D7))))&amp;""),$D7&amp;"")))</f>
+        <f>IF(AND($A7=""),"",IF(OR(($E7=""),($B7="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E7))*(EXACT('Asignacion'!$B$4:$B$34,$B7)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E7))*(EXACT('Asignacion'!$B$4:$B$34,$B7)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E7))*(EXACT('Asignacion'!$B$4:$B$34,$B7)),0),0))))))</f>
         <v/>
       </c>
       <c r="K7" s="3">
-        <f>IF(AND($A7=""),"",IF(EXACT($I7,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I7)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I7)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I7)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A7=""),"",IF(AND(NOT(EXACT($J7,"")),EXACT($J7,$I7)),1,0))</f>
         <v/>
       </c>
       <c r="L7" s="3">
-        <f>IF(AND($A7=""),"",IF(AND(NOT(EXACT($I7,"")),EXACT($K7,$J7)),1,0))</f>
+        <f>IF(AND($A7=""),"",MID(IF(AND(NOT(($B7="")),($E7="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M7" s="3">
-        <f>IF(AND($A7=""),"",MID(IF(AND(NOT(($B7="")),($E7="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N7" s="3">
         <f>IF(OR(AND(NOT(($B7="")),($E7=""))),2,0)</f>
         <v/>
       </c>
@@ -876,26 +854,22 @@
         <v/>
       </c>
       <c r="I8" s="3">
-        <f>IF(AND($A8=""),"",IF(OR(($E8=""),($B8="")),"",(IF(ISNUMBER($E8),IF($E8=0,"0",ROUND($E8,9-INT(LOG10(ABS($E8))))&amp;""),$E8&amp;"")&amp;"|"&amp;IF(ISNUMBER($B8),IF($B8=0,"0",ROUND($B8,9-INT(LOG10(ABS($B8))))&amp;""),$B8&amp;""))))</f>
+        <f>IF(AND($A8=""),"",(IF(ISNUMBER($B8),IF($B8=0,"0",ROUND($B8,9-INT(LOG10(ABS($B8))))&amp;""),$B8&amp;"")&amp;" "&amp;IF(ISNUMBER($C8),IF($C8=0,"0",ROUND($C8,9-INT(LOG10(ABS($C8))))&amp;""),$C8&amp;"")&amp;" "&amp;IF(ISNUMBER($D8),IF($D8=0,"0",ROUND($D8,9-INT(LOG10(ABS($D8))))&amp;""),$D8&amp;"")))</f>
         <v/>
       </c>
       <c r="J8" s="3">
-        <f>IF(AND($A8=""),"",(IF(ISNUMBER($B8),IF($B8=0,"0",ROUND($B8,9-INT(LOG10(ABS($B8))))&amp;""),$B8&amp;"")&amp;" "&amp;IF(ISNUMBER($C8),IF($C8=0,"0",ROUND($C8,9-INT(LOG10(ABS($C8))))&amp;""),$C8&amp;"")&amp;" "&amp;IF(ISNUMBER($D8),IF($D8=0,"0",ROUND($D8,9-INT(LOG10(ABS($D8))))&amp;""),$D8&amp;"")))</f>
+        <f>IF(AND($A8=""),"",IF(OR(($E8=""),($B8="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E8))*(EXACT('Asignacion'!$B$4:$B$34,$B8)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E8))*(EXACT('Asignacion'!$B$4:$B$34,$B8)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E8))*(EXACT('Asignacion'!$B$4:$B$34,$B8)),0),0))))))</f>
         <v/>
       </c>
       <c r="K8" s="3">
-        <f>IF(AND($A8=""),"",IF(EXACT($I8,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I8)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I8)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I8)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A8=""),"",IF(AND(NOT(EXACT($J8,"")),EXACT($J8,$I8)),1,0))</f>
         <v/>
       </c>
       <c r="L8" s="3">
-        <f>IF(AND($A8=""),"",IF(AND(NOT(EXACT($I8,"")),EXACT($K8,$J8)),1,0))</f>
+        <f>IF(AND($A8=""),"",MID(IF(AND(NOT(($B8="")),($E8="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M8" s="3">
-        <f>IF(AND($A8=""),"",MID(IF(AND(NOT(($B8="")),($E8="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N8" s="3">
         <f>IF(OR(AND(NOT(($B8="")),($E8=""))),2,0)</f>
         <v/>
       </c>
@@ -933,26 +907,22 @@
         <v/>
       </c>
       <c r="I9" s="3">
-        <f>IF(AND($A9=""),"",IF(OR(($E9=""),($B9="")),"",(IF(ISNUMBER($E9),IF($E9=0,"0",ROUND($E9,9-INT(LOG10(ABS($E9))))&amp;""),$E9&amp;"")&amp;"|"&amp;IF(ISNUMBER($B9),IF($B9=0,"0",ROUND($B9,9-INT(LOG10(ABS($B9))))&amp;""),$B9&amp;""))))</f>
+        <f>IF(AND($A9=""),"",(IF(ISNUMBER($B9),IF($B9=0,"0",ROUND($B9,9-INT(LOG10(ABS($B9))))&amp;""),$B9&amp;"")&amp;" "&amp;IF(ISNUMBER($C9),IF($C9=0,"0",ROUND($C9,9-INT(LOG10(ABS($C9))))&amp;""),$C9&amp;"")&amp;" "&amp;IF(ISNUMBER($D9),IF($D9=0,"0",ROUND($D9,9-INT(LOG10(ABS($D9))))&amp;""),$D9&amp;"")))</f>
         <v/>
       </c>
       <c r="J9" s="3">
-        <f>IF(AND($A9=""),"",(IF(ISNUMBER($B9),IF($B9=0,"0",ROUND($B9,9-INT(LOG10(ABS($B9))))&amp;""),$B9&amp;"")&amp;" "&amp;IF(ISNUMBER($C9),IF($C9=0,"0",ROUND($C9,9-INT(LOG10(ABS($C9))))&amp;""),$C9&amp;"")&amp;" "&amp;IF(ISNUMBER($D9),IF($D9=0,"0",ROUND($D9,9-INT(LOG10(ABS($D9))))&amp;""),$D9&amp;"")))</f>
+        <f>IF(AND($A9=""),"",IF(OR(($E9=""),($B9="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E9))*(EXACT('Asignacion'!$B$4:$B$34,$B9)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E9))*(EXACT('Asignacion'!$B$4:$B$34,$B9)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E9))*(EXACT('Asignacion'!$B$4:$B$34,$B9)),0),0))))))</f>
         <v/>
       </c>
       <c r="K9" s="3">
-        <f>IF(AND($A9=""),"",IF(EXACT($I9,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I9)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I9)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I9)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A9=""),"",IF(AND(NOT(EXACT($J9,"")),EXACT($J9,$I9)),1,0))</f>
         <v/>
       </c>
       <c r="L9" s="3">
-        <f>IF(AND($A9=""),"",IF(AND(NOT(EXACT($I9,"")),EXACT($K9,$J9)),1,0))</f>
+        <f>IF(AND($A9=""),"",MID(IF(AND(NOT(($B9="")),($E9="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M9" s="3">
-        <f>IF(AND($A9=""),"",MID(IF(AND(NOT(($B9="")),($E9="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N9" s="3">
         <f>IF(OR(AND(NOT(($B9="")),($E9=""))),2,0)</f>
         <v/>
       </c>
@@ -994,26 +964,22 @@
         <v/>
       </c>
       <c r="I10" s="3">
-        <f>IF(AND($A10=""),"",IF(OR(($E10=""),($B10="")),"",(IF(ISNUMBER($E10),IF($E10=0,"0",ROUND($E10,9-INT(LOG10(ABS($E10))))&amp;""),$E10&amp;"")&amp;"|"&amp;IF(ISNUMBER($B10),IF($B10=0,"0",ROUND($B10,9-INT(LOG10(ABS($B10))))&amp;""),$B10&amp;""))))</f>
+        <f>IF(AND($A10=""),"",(IF(ISNUMBER($B10),IF($B10=0,"0",ROUND($B10,9-INT(LOG10(ABS($B10))))&amp;""),$B10&amp;"")&amp;" "&amp;IF(ISNUMBER($C10),IF($C10=0,"0",ROUND($C10,9-INT(LOG10(ABS($C10))))&amp;""),$C10&amp;"")&amp;" "&amp;IF(ISNUMBER($D10),IF($D10=0,"0",ROUND($D10,9-INT(LOG10(ABS($D10))))&amp;""),$D10&amp;"")))</f>
         <v/>
       </c>
       <c r="J10" s="3">
-        <f>IF(AND($A10=""),"",(IF(ISNUMBER($B10),IF($B10=0,"0",ROUND($B10,9-INT(LOG10(ABS($B10))))&amp;""),$B10&amp;"")&amp;" "&amp;IF(ISNUMBER($C10),IF($C10=0,"0",ROUND($C10,9-INT(LOG10(ABS($C10))))&amp;""),$C10&amp;"")&amp;" "&amp;IF(ISNUMBER($D10),IF($D10=0,"0",ROUND($D10,9-INT(LOG10(ABS($D10))))&amp;""),$D10&amp;"")))</f>
+        <f>IF(AND($A10=""),"",IF(OR(($E10=""),($B10="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E10))*(EXACT('Asignacion'!$B$4:$B$34,$B10)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E10))*(EXACT('Asignacion'!$B$4:$B$34,$B10)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E10))*(EXACT('Asignacion'!$B$4:$B$34,$B10)),0),0))))))</f>
         <v/>
       </c>
       <c r="K10" s="3">
-        <f>IF(AND($A10=""),"",IF(EXACT($I10,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I10)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I10)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I10)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A10=""),"",IF(AND(NOT(EXACT($J10,"")),EXACT($J10,$I10)),1,0))</f>
         <v/>
       </c>
       <c r="L10" s="3">
-        <f>IF(AND($A10=""),"",IF(AND(NOT(EXACT($I10,"")),EXACT($K10,$J10)),1,0))</f>
+        <f>IF(AND($A10=""),"",MID(IF(AND(NOT(($B10="")),($E10="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M10" s="3">
-        <f>IF(AND($A10=""),"",MID(IF(AND(NOT(($B10="")),($E10="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N10" s="3">
         <f>IF(OR(AND(NOT(($B10="")),($E10=""))),2,0)</f>
         <v/>
       </c>
@@ -1051,26 +1017,22 @@
         <v/>
       </c>
       <c r="I11" s="3">
-        <f>IF(AND($A11=""),"",IF(OR(($E11=""),($B11="")),"",(IF(ISNUMBER($E11),IF($E11=0,"0",ROUND($E11,9-INT(LOG10(ABS($E11))))&amp;""),$E11&amp;"")&amp;"|"&amp;IF(ISNUMBER($B11),IF($B11=0,"0",ROUND($B11,9-INT(LOG10(ABS($B11))))&amp;""),$B11&amp;""))))</f>
+        <f>IF(AND($A11=""),"",(IF(ISNUMBER($B11),IF($B11=0,"0",ROUND($B11,9-INT(LOG10(ABS($B11))))&amp;""),$B11&amp;"")&amp;" "&amp;IF(ISNUMBER($C11),IF($C11=0,"0",ROUND($C11,9-INT(LOG10(ABS($C11))))&amp;""),$C11&amp;"")&amp;" "&amp;IF(ISNUMBER($D11),IF($D11=0,"0",ROUND($D11,9-INT(LOG10(ABS($D11))))&amp;""),$D11&amp;"")))</f>
         <v/>
       </c>
       <c r="J11" s="3">
-        <f>IF(AND($A11=""),"",(IF(ISNUMBER($B11),IF($B11=0,"0",ROUND($B11,9-INT(LOG10(ABS($B11))))&amp;""),$B11&amp;"")&amp;" "&amp;IF(ISNUMBER($C11),IF($C11=0,"0",ROUND($C11,9-INT(LOG10(ABS($C11))))&amp;""),$C11&amp;"")&amp;" "&amp;IF(ISNUMBER($D11),IF($D11=0,"0",ROUND($D11,9-INT(LOG10(ABS($D11))))&amp;""),$D11&amp;"")))</f>
+        <f>IF(AND($A11=""),"",IF(OR(($E11=""),($B11="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E11))*(EXACT('Asignacion'!$B$4:$B$34,$B11)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E11))*(EXACT('Asignacion'!$B$4:$B$34,$B11)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E11))*(EXACT('Asignacion'!$B$4:$B$34,$B11)),0),0))))))</f>
         <v/>
       </c>
       <c r="K11" s="3">
-        <f>IF(AND($A11=""),"",IF(EXACT($I11,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I11)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I11)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I11)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A11=""),"",IF(AND(NOT(EXACT($J11,"")),EXACT($J11,$I11)),1,0))</f>
         <v/>
       </c>
       <c r="L11" s="3">
-        <f>IF(AND($A11=""),"",IF(AND(NOT(EXACT($I11,"")),EXACT($K11,$J11)),1,0))</f>
+        <f>IF(AND($A11=""),"",MID(IF(AND(NOT(($B11="")),($E11="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M11" s="3">
-        <f>IF(AND($A11=""),"",MID(IF(AND(NOT(($B11="")),($E11="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N11" s="3">
         <f>IF(OR(AND(NOT(($B11="")),($E11=""))),2,0)</f>
         <v/>
       </c>
@@ -1108,26 +1070,22 @@
         <v/>
       </c>
       <c r="I12" s="3">
-        <f>IF(AND($A12=""),"",IF(OR(($E12=""),($B12="")),"",(IF(ISNUMBER($E12),IF($E12=0,"0",ROUND($E12,9-INT(LOG10(ABS($E12))))&amp;""),$E12&amp;"")&amp;"|"&amp;IF(ISNUMBER($B12),IF($B12=0,"0",ROUND($B12,9-INT(LOG10(ABS($B12))))&amp;""),$B12&amp;""))))</f>
+        <f>IF(AND($A12=""),"",(IF(ISNUMBER($B12),IF($B12=0,"0",ROUND($B12,9-INT(LOG10(ABS($B12))))&amp;""),$B12&amp;"")&amp;" "&amp;IF(ISNUMBER($C12),IF($C12=0,"0",ROUND($C12,9-INT(LOG10(ABS($C12))))&amp;""),$C12&amp;"")&amp;" "&amp;IF(ISNUMBER($D12),IF($D12=0,"0",ROUND($D12,9-INT(LOG10(ABS($D12))))&amp;""),$D12&amp;"")))</f>
         <v/>
       </c>
       <c r="J12" s="3">
-        <f>IF(AND($A12=""),"",(IF(ISNUMBER($B12),IF($B12=0,"0",ROUND($B12,9-INT(LOG10(ABS($B12))))&amp;""),$B12&amp;"")&amp;" "&amp;IF(ISNUMBER($C12),IF($C12=0,"0",ROUND($C12,9-INT(LOG10(ABS($C12))))&amp;""),$C12&amp;"")&amp;" "&amp;IF(ISNUMBER($D12),IF($D12=0,"0",ROUND($D12,9-INT(LOG10(ABS($D12))))&amp;""),$D12&amp;"")))</f>
+        <f>IF(AND($A12=""),"",IF(OR(($E12=""),($B12="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E12))*(EXACT('Asignacion'!$B$4:$B$34,$B12)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E12))*(EXACT('Asignacion'!$B$4:$B$34,$B12)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E12))*(EXACT('Asignacion'!$B$4:$B$34,$B12)),0),0))))))</f>
         <v/>
       </c>
       <c r="K12" s="3">
-        <f>IF(AND($A12=""),"",IF(EXACT($I12,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I12)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I12)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I12)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A12=""),"",IF(AND(NOT(EXACT($J12,"")),EXACT($J12,$I12)),1,0))</f>
         <v/>
       </c>
       <c r="L12" s="3">
-        <f>IF(AND($A12=""),"",IF(AND(NOT(EXACT($I12,"")),EXACT($K12,$J12)),1,0))</f>
+        <f>IF(AND($A12=""),"",MID(IF(AND(NOT(($B12="")),($E12="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M12" s="3">
-        <f>IF(AND($A12=""),"",MID(IF(AND(NOT(($B12="")),($E12="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N12" s="3">
         <f>IF(OR(AND(NOT(($B12="")),($E12=""))),2,0)</f>
         <v/>
       </c>
@@ -1153,26 +1111,22 @@
         <v/>
       </c>
       <c r="I13" s="3">
-        <f>IF(AND($A13=""),"",IF(OR(($E13=""),($B13="")),"",(IF(ISNUMBER($E13),IF($E13=0,"0",ROUND($E13,9-INT(LOG10(ABS($E13))))&amp;""),$E13&amp;"")&amp;"|"&amp;IF(ISNUMBER($B13),IF($B13=0,"0",ROUND($B13,9-INT(LOG10(ABS($B13))))&amp;""),$B13&amp;""))))</f>
+        <f>IF(AND($A13=""),"",(IF(ISNUMBER($B13),IF($B13=0,"0",ROUND($B13,9-INT(LOG10(ABS($B13))))&amp;""),$B13&amp;"")&amp;" "&amp;IF(ISNUMBER($C13),IF($C13=0,"0",ROUND($C13,9-INT(LOG10(ABS($C13))))&amp;""),$C13&amp;"")&amp;" "&amp;IF(ISNUMBER($D13),IF($D13=0,"0",ROUND($D13,9-INT(LOG10(ABS($D13))))&amp;""),$D13&amp;"")))</f>
         <v/>
       </c>
       <c r="J13" s="3">
-        <f>IF(AND($A13=""),"",(IF(ISNUMBER($B13),IF($B13=0,"0",ROUND($B13,9-INT(LOG10(ABS($B13))))&amp;""),$B13&amp;"")&amp;" "&amp;IF(ISNUMBER($C13),IF($C13=0,"0",ROUND($C13,9-INT(LOG10(ABS($C13))))&amp;""),$C13&amp;"")&amp;" "&amp;IF(ISNUMBER($D13),IF($D13=0,"0",ROUND($D13,9-INT(LOG10(ABS($D13))))&amp;""),$D13&amp;"")))</f>
+        <f>IF(AND($A13=""),"",IF(OR(($E13=""),($B13="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E13))*(EXACT('Asignacion'!$B$4:$B$34,$B13)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E13))*(EXACT('Asignacion'!$B$4:$B$34,$B13)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E13))*(EXACT('Asignacion'!$B$4:$B$34,$B13)),0),0))))))</f>
         <v/>
       </c>
       <c r="K13" s="3">
-        <f>IF(AND($A13=""),"",IF(EXACT($I13,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I13)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I13)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I13)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A13=""),"",IF(AND(NOT(EXACT($J13,"")),EXACT($J13,$I13)),1,0))</f>
         <v/>
       </c>
       <c r="L13" s="3">
-        <f>IF(AND($A13=""),"",IF(AND(NOT(EXACT($I13,"")),EXACT($K13,$J13)),1,0))</f>
+        <f>IF(AND($A13=""),"",MID(IF(AND(NOT(($B13="")),($E13="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M13" s="3">
-        <f>IF(AND($A13=""),"",MID(IF(AND(NOT(($B13="")),($E13="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N13" s="3">
         <f>IF(OR(AND(NOT(($B13="")),($E13=""))),2,0)</f>
         <v/>
       </c>
@@ -1198,26 +1152,22 @@
         <v/>
       </c>
       <c r="I14" s="3">
-        <f>IF(AND($A14=""),"",IF(OR(($E14=""),($B14="")),"",(IF(ISNUMBER($E14),IF($E14=0,"0",ROUND($E14,9-INT(LOG10(ABS($E14))))&amp;""),$E14&amp;"")&amp;"|"&amp;IF(ISNUMBER($B14),IF($B14=0,"0",ROUND($B14,9-INT(LOG10(ABS($B14))))&amp;""),$B14&amp;""))))</f>
+        <f>IF(AND($A14=""),"",(IF(ISNUMBER($B14),IF($B14=0,"0",ROUND($B14,9-INT(LOG10(ABS($B14))))&amp;""),$B14&amp;"")&amp;" "&amp;IF(ISNUMBER($C14),IF($C14=0,"0",ROUND($C14,9-INT(LOG10(ABS($C14))))&amp;""),$C14&amp;"")&amp;" "&amp;IF(ISNUMBER($D14),IF($D14=0,"0",ROUND($D14,9-INT(LOG10(ABS($D14))))&amp;""),$D14&amp;"")))</f>
         <v/>
       </c>
       <c r="J14" s="3">
-        <f>IF(AND($A14=""),"",(IF(ISNUMBER($B14),IF($B14=0,"0",ROUND($B14,9-INT(LOG10(ABS($B14))))&amp;""),$B14&amp;"")&amp;" "&amp;IF(ISNUMBER($C14),IF($C14=0,"0",ROUND($C14,9-INT(LOG10(ABS($C14))))&amp;""),$C14&amp;"")&amp;" "&amp;IF(ISNUMBER($D14),IF($D14=0,"0",ROUND($D14,9-INT(LOG10(ABS($D14))))&amp;""),$D14&amp;"")))</f>
+        <f>IF(AND($A14=""),"",IF(OR(($E14=""),($B14="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E14))*(EXACT('Asignacion'!$B$4:$B$34,$B14)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E14))*(EXACT('Asignacion'!$B$4:$B$34,$B14)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E14))*(EXACT('Asignacion'!$B$4:$B$34,$B14)),0),0))))))</f>
         <v/>
       </c>
       <c r="K14" s="3">
-        <f>IF(AND($A14=""),"",IF(EXACT($I14,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I14)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I14)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I14)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A14=""),"",IF(AND(NOT(EXACT($J14,"")),EXACT($J14,$I14)),1,0))</f>
         <v/>
       </c>
       <c r="L14" s="3">
-        <f>IF(AND($A14=""),"",IF(AND(NOT(EXACT($I14,"")),EXACT($K14,$J14)),1,0))</f>
+        <f>IF(AND($A14=""),"",MID(IF(AND(NOT(($B14="")),($E14="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M14" s="3">
-        <f>IF(AND($A14=""),"",MID(IF(AND(NOT(($B14="")),($E14="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N14" s="3">
         <f>IF(OR(AND(NOT(($B14="")),($E14=""))),2,0)</f>
         <v/>
       </c>
@@ -1241,26 +1191,22 @@
         <v/>
       </c>
       <c r="I15" s="3">
-        <f>IF(AND($A15=""),"",IF(OR(($E15=""),($B15="")),"",(IF(ISNUMBER($E15),IF($E15=0,"0",ROUND($E15,9-INT(LOG10(ABS($E15))))&amp;""),$E15&amp;"")&amp;"|"&amp;IF(ISNUMBER($B15),IF($B15=0,"0",ROUND($B15,9-INT(LOG10(ABS($B15))))&amp;""),$B15&amp;""))))</f>
+        <f>IF(AND($A15=""),"",(IF(ISNUMBER($B15),IF($B15=0,"0",ROUND($B15,9-INT(LOG10(ABS($B15))))&amp;""),$B15&amp;"")&amp;" "&amp;IF(ISNUMBER($C15),IF($C15=0,"0",ROUND($C15,9-INT(LOG10(ABS($C15))))&amp;""),$C15&amp;"")&amp;" "&amp;IF(ISNUMBER($D15),IF($D15=0,"0",ROUND($D15,9-INT(LOG10(ABS($D15))))&amp;""),$D15&amp;"")))</f>
         <v/>
       </c>
       <c r="J15" s="3">
-        <f>IF(AND($A15=""),"",(IF(ISNUMBER($B15),IF($B15=0,"0",ROUND($B15,9-INT(LOG10(ABS($B15))))&amp;""),$B15&amp;"")&amp;" "&amp;IF(ISNUMBER($C15),IF($C15=0,"0",ROUND($C15,9-INT(LOG10(ABS($C15))))&amp;""),$C15&amp;"")&amp;" "&amp;IF(ISNUMBER($D15),IF($D15=0,"0",ROUND($D15,9-INT(LOG10(ABS($D15))))&amp;""),$D15&amp;"")))</f>
+        <f>IF(AND($A15=""),"",IF(OR(($E15=""),($B15="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E15))*(EXACT('Asignacion'!$B$4:$B$34,$B15)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E15))*(EXACT('Asignacion'!$B$4:$B$34,$B15)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E15))*(EXACT('Asignacion'!$B$4:$B$34,$B15)),0),0))))))</f>
         <v/>
       </c>
       <c r="K15" s="3">
-        <f>IF(AND($A15=""),"",IF(EXACT($I15,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I15)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I15)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I15)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A15=""),"",IF(AND(NOT(EXACT($J15,"")),EXACT($J15,$I15)),1,0))</f>
         <v/>
       </c>
       <c r="L15" s="3">
-        <f>IF(AND($A15=""),"",IF(AND(NOT(EXACT($I15,"")),EXACT($K15,$J15)),1,0))</f>
+        <f>IF(AND($A15=""),"",MID(IF(AND(NOT(($B15="")),($E15="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M15" s="3">
-        <f>IF(AND($A15=""),"",MID(IF(AND(NOT(($B15="")),($E15="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N15" s="3">
         <f>IF(OR(AND(NOT(($B15="")),($E15=""))),2,0)</f>
         <v/>
       </c>
@@ -1284,26 +1230,22 @@
         <v/>
       </c>
       <c r="I16" s="3">
-        <f>IF(AND($A16=""),"",IF(OR(($E16=""),($B16="")),"",(IF(ISNUMBER($E16),IF($E16=0,"0",ROUND($E16,9-INT(LOG10(ABS($E16))))&amp;""),$E16&amp;"")&amp;"|"&amp;IF(ISNUMBER($B16),IF($B16=0,"0",ROUND($B16,9-INT(LOG10(ABS($B16))))&amp;""),$B16&amp;""))))</f>
+        <f>IF(AND($A16=""),"",(IF(ISNUMBER($B16),IF($B16=0,"0",ROUND($B16,9-INT(LOG10(ABS($B16))))&amp;""),$B16&amp;"")&amp;" "&amp;IF(ISNUMBER($C16),IF($C16=0,"0",ROUND($C16,9-INT(LOG10(ABS($C16))))&amp;""),$C16&amp;"")&amp;" "&amp;IF(ISNUMBER($D16),IF($D16=0,"0",ROUND($D16,9-INT(LOG10(ABS($D16))))&amp;""),$D16&amp;"")))</f>
         <v/>
       </c>
       <c r="J16" s="3">
-        <f>IF(AND($A16=""),"",(IF(ISNUMBER($B16),IF($B16=0,"0",ROUND($B16,9-INT(LOG10(ABS($B16))))&amp;""),$B16&amp;"")&amp;" "&amp;IF(ISNUMBER($C16),IF($C16=0,"0",ROUND($C16,9-INT(LOG10(ABS($C16))))&amp;""),$C16&amp;"")&amp;" "&amp;IF(ISNUMBER($D16),IF($D16=0,"0",ROUND($D16,9-INT(LOG10(ABS($D16))))&amp;""),$D16&amp;"")))</f>
+        <f>IF(AND($A16=""),"",IF(OR(($E16=""),($B16="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E16))*(EXACT('Asignacion'!$B$4:$B$34,$B16)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E16))*(EXACT('Asignacion'!$B$4:$B$34,$B16)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E16))*(EXACT('Asignacion'!$B$4:$B$34,$B16)),0),0))))))</f>
         <v/>
       </c>
       <c r="K16" s="3">
-        <f>IF(AND($A16=""),"",IF(EXACT($I16,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I16)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I16)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I16)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A16=""),"",IF(AND(NOT(EXACT($J16,"")),EXACT($J16,$I16)),1,0))</f>
         <v/>
       </c>
       <c r="L16" s="3">
-        <f>IF(AND($A16=""),"",IF(AND(NOT(EXACT($I16,"")),EXACT($K16,$J16)),1,0))</f>
+        <f>IF(AND($A16=""),"",MID(IF(AND(NOT(($B16="")),($E16="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M16" s="3">
-        <f>IF(AND($A16=""),"",MID(IF(AND(NOT(($B16="")),($E16="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N16" s="3">
         <f>IF(OR(AND(NOT(($B16="")),($E16=""))),2,0)</f>
         <v/>
       </c>
@@ -1327,26 +1269,22 @@
         <v/>
       </c>
       <c r="I17" s="3">
-        <f>IF(AND($A17=""),"",IF(OR(($E17=""),($B17="")),"",(IF(ISNUMBER($E17),IF($E17=0,"0",ROUND($E17,9-INT(LOG10(ABS($E17))))&amp;""),$E17&amp;"")&amp;"|"&amp;IF(ISNUMBER($B17),IF($B17=0,"0",ROUND($B17,9-INT(LOG10(ABS($B17))))&amp;""),$B17&amp;""))))</f>
+        <f>IF(AND($A17=""),"",(IF(ISNUMBER($B17),IF($B17=0,"0",ROUND($B17,9-INT(LOG10(ABS($B17))))&amp;""),$B17&amp;"")&amp;" "&amp;IF(ISNUMBER($C17),IF($C17=0,"0",ROUND($C17,9-INT(LOG10(ABS($C17))))&amp;""),$C17&amp;"")&amp;" "&amp;IF(ISNUMBER($D17),IF($D17=0,"0",ROUND($D17,9-INT(LOG10(ABS($D17))))&amp;""),$D17&amp;"")))</f>
         <v/>
       </c>
       <c r="J17" s="3">
-        <f>IF(AND($A17=""),"",(IF(ISNUMBER($B17),IF($B17=0,"0",ROUND($B17,9-INT(LOG10(ABS($B17))))&amp;""),$B17&amp;"")&amp;" "&amp;IF(ISNUMBER($C17),IF($C17=0,"0",ROUND($C17,9-INT(LOG10(ABS($C17))))&amp;""),$C17&amp;"")&amp;" "&amp;IF(ISNUMBER($D17),IF($D17=0,"0",ROUND($D17,9-INT(LOG10(ABS($D17))))&amp;""),$D17&amp;"")))</f>
+        <f>IF(AND($A17=""),"",IF(OR(($E17=""),($B17="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E17))*(EXACT('Asignacion'!$B$4:$B$34,$B17)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E17))*(EXACT('Asignacion'!$B$4:$B$34,$B17)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E17))*(EXACT('Asignacion'!$B$4:$B$34,$B17)),0),0))))))</f>
         <v/>
       </c>
       <c r="K17" s="3">
-        <f>IF(AND($A17=""),"",IF(EXACT($I17,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I17)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I17)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I17)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A17=""),"",IF(AND(NOT(EXACT($J17,"")),EXACT($J17,$I17)),1,0))</f>
         <v/>
       </c>
       <c r="L17" s="3">
-        <f>IF(AND($A17=""),"",IF(AND(NOT(EXACT($I17,"")),EXACT($K17,$J17)),1,0))</f>
+        <f>IF(AND($A17=""),"",MID(IF(AND(NOT(($B17="")),($E17="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M17" s="3">
-        <f>IF(AND($A17=""),"",MID(IF(AND(NOT(($B17="")),($E17="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N17" s="3">
         <f>IF(OR(AND(NOT(($B17="")),($E17=""))),2,0)</f>
         <v/>
       </c>
@@ -1370,26 +1308,22 @@
         <v/>
       </c>
       <c r="I18" s="3">
-        <f>IF(AND($A18=""),"",IF(OR(($E18=""),($B18="")),"",(IF(ISNUMBER($E18),IF($E18=0,"0",ROUND($E18,9-INT(LOG10(ABS($E18))))&amp;""),$E18&amp;"")&amp;"|"&amp;IF(ISNUMBER($B18),IF($B18=0,"0",ROUND($B18,9-INT(LOG10(ABS($B18))))&amp;""),$B18&amp;""))))</f>
+        <f>IF(AND($A18=""),"",(IF(ISNUMBER($B18),IF($B18=0,"0",ROUND($B18,9-INT(LOG10(ABS($B18))))&amp;""),$B18&amp;"")&amp;" "&amp;IF(ISNUMBER($C18),IF($C18=0,"0",ROUND($C18,9-INT(LOG10(ABS($C18))))&amp;""),$C18&amp;"")&amp;" "&amp;IF(ISNUMBER($D18),IF($D18=0,"0",ROUND($D18,9-INT(LOG10(ABS($D18))))&amp;""),$D18&amp;"")))</f>
         <v/>
       </c>
       <c r="J18" s="3">
-        <f>IF(AND($A18=""),"",(IF(ISNUMBER($B18),IF($B18=0,"0",ROUND($B18,9-INT(LOG10(ABS($B18))))&amp;""),$B18&amp;"")&amp;" "&amp;IF(ISNUMBER($C18),IF($C18=0,"0",ROUND($C18,9-INT(LOG10(ABS($C18))))&amp;""),$C18&amp;"")&amp;" "&amp;IF(ISNUMBER($D18),IF($D18=0,"0",ROUND($D18,9-INT(LOG10(ABS($D18))))&amp;""),$D18&amp;"")))</f>
+        <f>IF(AND($A18=""),"",IF(OR(($E18=""),($B18="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E18))*(EXACT('Asignacion'!$B$4:$B$34,$B18)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E18))*(EXACT('Asignacion'!$B$4:$B$34,$B18)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E18))*(EXACT('Asignacion'!$B$4:$B$34,$B18)),0),0))))))</f>
         <v/>
       </c>
       <c r="K18" s="3">
-        <f>IF(AND($A18=""),"",IF(EXACT($I18,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I18)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I18)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I18)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A18=""),"",IF(AND(NOT(EXACT($J18,"")),EXACT($J18,$I18)),1,0))</f>
         <v/>
       </c>
       <c r="L18" s="3">
-        <f>IF(AND($A18=""),"",IF(AND(NOT(EXACT($I18,"")),EXACT($K18,$J18)),1,0))</f>
+        <f>IF(AND($A18=""),"",MID(IF(AND(NOT(($B18="")),($E18="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M18" s="3">
-        <f>IF(AND($A18=""),"",MID(IF(AND(NOT(($B18="")),($E18="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N18" s="3">
         <f>IF(OR(AND(NOT(($B18="")),($E18=""))),2,0)</f>
         <v/>
       </c>
@@ -1413,26 +1347,22 @@
         <v/>
       </c>
       <c r="I19" s="3">
-        <f>IF(AND($A19=""),"",IF(OR(($E19=""),($B19="")),"",(IF(ISNUMBER($E19),IF($E19=0,"0",ROUND($E19,9-INT(LOG10(ABS($E19))))&amp;""),$E19&amp;"")&amp;"|"&amp;IF(ISNUMBER($B19),IF($B19=0,"0",ROUND($B19,9-INT(LOG10(ABS($B19))))&amp;""),$B19&amp;""))))</f>
+        <f>IF(AND($A19=""),"",(IF(ISNUMBER($B19),IF($B19=0,"0",ROUND($B19,9-INT(LOG10(ABS($B19))))&amp;""),$B19&amp;"")&amp;" "&amp;IF(ISNUMBER($C19),IF($C19=0,"0",ROUND($C19,9-INT(LOG10(ABS($C19))))&amp;""),$C19&amp;"")&amp;" "&amp;IF(ISNUMBER($D19),IF($D19=0,"0",ROUND($D19,9-INT(LOG10(ABS($D19))))&amp;""),$D19&amp;"")))</f>
         <v/>
       </c>
       <c r="J19" s="3">
-        <f>IF(AND($A19=""),"",(IF(ISNUMBER($B19),IF($B19=0,"0",ROUND($B19,9-INT(LOG10(ABS($B19))))&amp;""),$B19&amp;"")&amp;" "&amp;IF(ISNUMBER($C19),IF($C19=0,"0",ROUND($C19,9-INT(LOG10(ABS($C19))))&amp;""),$C19&amp;"")&amp;" "&amp;IF(ISNUMBER($D19),IF($D19=0,"0",ROUND($D19,9-INT(LOG10(ABS($D19))))&amp;""),$D19&amp;"")))</f>
+        <f>IF(AND($A19=""),"",IF(OR(($E19=""),($B19="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E19))*(EXACT('Asignacion'!$B$4:$B$34,$B19)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E19))*(EXACT('Asignacion'!$B$4:$B$34,$B19)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E19))*(EXACT('Asignacion'!$B$4:$B$34,$B19)),0),0))))))</f>
         <v/>
       </c>
       <c r="K19" s="3">
-        <f>IF(AND($A19=""),"",IF(EXACT($I19,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I19)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I19)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I19)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A19=""),"",IF(AND(NOT(EXACT($J19,"")),EXACT($J19,$I19)),1,0))</f>
         <v/>
       </c>
       <c r="L19" s="3">
-        <f>IF(AND($A19=""),"",IF(AND(NOT(EXACT($I19,"")),EXACT($K19,$J19)),1,0))</f>
+        <f>IF(AND($A19=""),"",MID(IF(AND(NOT(($B19="")),($E19="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M19" s="3">
-        <f>IF(AND($A19=""),"",MID(IF(AND(NOT(($B19="")),($E19="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N19" s="3">
         <f>IF(OR(AND(NOT(($B19="")),($E19=""))),2,0)</f>
         <v/>
       </c>
@@ -1456,26 +1386,22 @@
         <v/>
       </c>
       <c r="I20" s="3">
-        <f>IF(AND($A20=""),"",IF(OR(($E20=""),($B20="")),"",(IF(ISNUMBER($E20),IF($E20=0,"0",ROUND($E20,9-INT(LOG10(ABS($E20))))&amp;""),$E20&amp;"")&amp;"|"&amp;IF(ISNUMBER($B20),IF($B20=0,"0",ROUND($B20,9-INT(LOG10(ABS($B20))))&amp;""),$B20&amp;""))))</f>
+        <f>IF(AND($A20=""),"",(IF(ISNUMBER($B20),IF($B20=0,"0",ROUND($B20,9-INT(LOG10(ABS($B20))))&amp;""),$B20&amp;"")&amp;" "&amp;IF(ISNUMBER($C20),IF($C20=0,"0",ROUND($C20,9-INT(LOG10(ABS($C20))))&amp;""),$C20&amp;"")&amp;" "&amp;IF(ISNUMBER($D20),IF($D20=0,"0",ROUND($D20,9-INT(LOG10(ABS($D20))))&amp;""),$D20&amp;"")))</f>
         <v/>
       </c>
       <c r="J20" s="3">
-        <f>IF(AND($A20=""),"",(IF(ISNUMBER($B20),IF($B20=0,"0",ROUND($B20,9-INT(LOG10(ABS($B20))))&amp;""),$B20&amp;"")&amp;" "&amp;IF(ISNUMBER($C20),IF($C20=0,"0",ROUND($C20,9-INT(LOG10(ABS($C20))))&amp;""),$C20&amp;"")&amp;" "&amp;IF(ISNUMBER($D20),IF($D20=0,"0",ROUND($D20,9-INT(LOG10(ABS($D20))))&amp;""),$D20&amp;"")))</f>
+        <f>IF(AND($A20=""),"",IF(OR(($E20=""),($B20="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E20))*(EXACT('Asignacion'!$B$4:$B$34,$B20)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E20))*(EXACT('Asignacion'!$B$4:$B$34,$B20)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E20))*(EXACT('Asignacion'!$B$4:$B$34,$B20)),0),0))))))</f>
         <v/>
       </c>
       <c r="K20" s="3">
-        <f>IF(AND($A20=""),"",IF(EXACT($I20,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I20)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I20)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I20)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A20=""),"",IF(AND(NOT(EXACT($J20,"")),EXACT($J20,$I20)),1,0))</f>
         <v/>
       </c>
       <c r="L20" s="3">
-        <f>IF(AND($A20=""),"",IF(AND(NOT(EXACT($I20,"")),EXACT($K20,$J20)),1,0))</f>
+        <f>IF(AND($A20=""),"",MID(IF(AND(NOT(($B20="")),($E20="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M20" s="3">
-        <f>IF(AND($A20=""),"",MID(IF(AND(NOT(($B20="")),($E20="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N20" s="3">
         <f>IF(OR(AND(NOT(($B20="")),($E20=""))),2,0)</f>
         <v/>
       </c>
@@ -1499,26 +1425,22 @@
         <v/>
       </c>
       <c r="I21" s="3">
-        <f>IF(AND($A21=""),"",IF(OR(($E21=""),($B21="")),"",(IF(ISNUMBER($E21),IF($E21=0,"0",ROUND($E21,9-INT(LOG10(ABS($E21))))&amp;""),$E21&amp;"")&amp;"|"&amp;IF(ISNUMBER($B21),IF($B21=0,"0",ROUND($B21,9-INT(LOG10(ABS($B21))))&amp;""),$B21&amp;""))))</f>
+        <f>IF(AND($A21=""),"",(IF(ISNUMBER($B21),IF($B21=0,"0",ROUND($B21,9-INT(LOG10(ABS($B21))))&amp;""),$B21&amp;"")&amp;" "&amp;IF(ISNUMBER($C21),IF($C21=0,"0",ROUND($C21,9-INT(LOG10(ABS($C21))))&amp;""),$C21&amp;"")&amp;" "&amp;IF(ISNUMBER($D21),IF($D21=0,"0",ROUND($D21,9-INT(LOG10(ABS($D21))))&amp;""),$D21&amp;"")))</f>
         <v/>
       </c>
       <c r="J21" s="3">
-        <f>IF(AND($A21=""),"",(IF(ISNUMBER($B21),IF($B21=0,"0",ROUND($B21,9-INT(LOG10(ABS($B21))))&amp;""),$B21&amp;"")&amp;" "&amp;IF(ISNUMBER($C21),IF($C21=0,"0",ROUND($C21,9-INT(LOG10(ABS($C21))))&amp;""),$C21&amp;"")&amp;" "&amp;IF(ISNUMBER($D21),IF($D21=0,"0",ROUND($D21,9-INT(LOG10(ABS($D21))))&amp;""),$D21&amp;"")))</f>
+        <f>IF(AND($A21=""),"",IF(OR(($E21=""),($B21="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E21))*(EXACT('Asignacion'!$B$4:$B$34,$B21)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E21))*(EXACT('Asignacion'!$B$4:$B$34,$B21)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E21))*(EXACT('Asignacion'!$B$4:$B$34,$B21)),0),0))))))</f>
         <v/>
       </c>
       <c r="K21" s="3">
-        <f>IF(AND($A21=""),"",IF(EXACT($I21,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I21)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I21)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I21)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A21=""),"",IF(AND(NOT(EXACT($J21,"")),EXACT($J21,$I21)),1,0))</f>
         <v/>
       </c>
       <c r="L21" s="3">
-        <f>IF(AND($A21=""),"",IF(AND(NOT(EXACT($I21,"")),EXACT($K21,$J21)),1,0))</f>
+        <f>IF(AND($A21=""),"",MID(IF(AND(NOT(($B21="")),($E21="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M21" s="3">
-        <f>IF(AND($A21=""),"",MID(IF(AND(NOT(($B21="")),($E21="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N21" s="3">
         <f>IF(OR(AND(NOT(($B21="")),($E21=""))),2,0)</f>
         <v/>
       </c>
@@ -1542,26 +1464,22 @@
         <v/>
       </c>
       <c r="I22" s="3">
-        <f>IF(AND($A22=""),"",IF(OR(($E22=""),($B22="")),"",(IF(ISNUMBER($E22),IF($E22=0,"0",ROUND($E22,9-INT(LOG10(ABS($E22))))&amp;""),$E22&amp;"")&amp;"|"&amp;IF(ISNUMBER($B22),IF($B22=0,"0",ROUND($B22,9-INT(LOG10(ABS($B22))))&amp;""),$B22&amp;""))))</f>
+        <f>IF(AND($A22=""),"",(IF(ISNUMBER($B22),IF($B22=0,"0",ROUND($B22,9-INT(LOG10(ABS($B22))))&amp;""),$B22&amp;"")&amp;" "&amp;IF(ISNUMBER($C22),IF($C22=0,"0",ROUND($C22,9-INT(LOG10(ABS($C22))))&amp;""),$C22&amp;"")&amp;" "&amp;IF(ISNUMBER($D22),IF($D22=0,"0",ROUND($D22,9-INT(LOG10(ABS($D22))))&amp;""),$D22&amp;"")))</f>
         <v/>
       </c>
       <c r="J22" s="3">
-        <f>IF(AND($A22=""),"",(IF(ISNUMBER($B22),IF($B22=0,"0",ROUND($B22,9-INT(LOG10(ABS($B22))))&amp;""),$B22&amp;"")&amp;" "&amp;IF(ISNUMBER($C22),IF($C22=0,"0",ROUND($C22,9-INT(LOG10(ABS($C22))))&amp;""),$C22&amp;"")&amp;" "&amp;IF(ISNUMBER($D22),IF($D22=0,"0",ROUND($D22,9-INT(LOG10(ABS($D22))))&amp;""),$D22&amp;"")))</f>
+        <f>IF(AND($A22=""),"",IF(OR(($E22=""),($B22="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E22))*(EXACT('Asignacion'!$B$4:$B$34,$B22)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E22))*(EXACT('Asignacion'!$B$4:$B$34,$B22)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E22))*(EXACT('Asignacion'!$B$4:$B$34,$B22)),0),0))))))</f>
         <v/>
       </c>
       <c r="K22" s="3">
-        <f>IF(AND($A22=""),"",IF(EXACT($I22,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I22)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I22)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I22)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A22=""),"",IF(AND(NOT(EXACT($J22,"")),EXACT($J22,$I22)),1,0))</f>
         <v/>
       </c>
       <c r="L22" s="3">
-        <f>IF(AND($A22=""),"",IF(AND(NOT(EXACT($I22,"")),EXACT($K22,$J22)),1,0))</f>
+        <f>IF(AND($A22=""),"",MID(IF(AND(NOT(($B22="")),($E22="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M22" s="3">
-        <f>IF(AND($A22=""),"",MID(IF(AND(NOT(($B22="")),($E22="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N22" s="3">
         <f>IF(OR(AND(NOT(($B22="")),($E22=""))),2,0)</f>
         <v/>
       </c>
@@ -1585,26 +1503,22 @@
         <v/>
       </c>
       <c r="I23" s="3">
-        <f>IF(AND($A23=""),"",IF(OR(($E23=""),($B23="")),"",(IF(ISNUMBER($E23),IF($E23=0,"0",ROUND($E23,9-INT(LOG10(ABS($E23))))&amp;""),$E23&amp;"")&amp;"|"&amp;IF(ISNUMBER($B23),IF($B23=0,"0",ROUND($B23,9-INT(LOG10(ABS($B23))))&amp;""),$B23&amp;""))))</f>
+        <f>IF(AND($A23=""),"",(IF(ISNUMBER($B23),IF($B23=0,"0",ROUND($B23,9-INT(LOG10(ABS($B23))))&amp;""),$B23&amp;"")&amp;" "&amp;IF(ISNUMBER($C23),IF($C23=0,"0",ROUND($C23,9-INT(LOG10(ABS($C23))))&amp;""),$C23&amp;"")&amp;" "&amp;IF(ISNUMBER($D23),IF($D23=0,"0",ROUND($D23,9-INT(LOG10(ABS($D23))))&amp;""),$D23&amp;"")))</f>
         <v/>
       </c>
       <c r="J23" s="3">
-        <f>IF(AND($A23=""),"",(IF(ISNUMBER($B23),IF($B23=0,"0",ROUND($B23,9-INT(LOG10(ABS($B23))))&amp;""),$B23&amp;"")&amp;" "&amp;IF(ISNUMBER($C23),IF($C23=0,"0",ROUND($C23,9-INT(LOG10(ABS($C23))))&amp;""),$C23&amp;"")&amp;" "&amp;IF(ISNUMBER($D23),IF($D23=0,"0",ROUND($D23,9-INT(LOG10(ABS($D23))))&amp;""),$D23&amp;"")))</f>
+        <f>IF(AND($A23=""),"",IF(OR(($E23=""),($B23="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E23))*(EXACT('Asignacion'!$B$4:$B$34,$B23)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E23))*(EXACT('Asignacion'!$B$4:$B$34,$B23)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E23))*(EXACT('Asignacion'!$B$4:$B$34,$B23)),0),0))))))</f>
         <v/>
       </c>
       <c r="K23" s="3">
-        <f>IF(AND($A23=""),"",IF(EXACT($I23,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I23)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I23)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I23)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A23=""),"",IF(AND(NOT(EXACT($J23,"")),EXACT($J23,$I23)),1,0))</f>
         <v/>
       </c>
       <c r="L23" s="3">
-        <f>IF(AND($A23=""),"",IF(AND(NOT(EXACT($I23,"")),EXACT($K23,$J23)),1,0))</f>
+        <f>IF(AND($A23=""),"",MID(IF(AND(NOT(($B23="")),($E23="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M23" s="3">
-        <f>IF(AND($A23=""),"",MID(IF(AND(NOT(($B23="")),($E23="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N23" s="3">
         <f>IF(OR(AND(NOT(($B23="")),($E23=""))),2,0)</f>
         <v/>
       </c>
@@ -1628,26 +1542,22 @@
         <v/>
       </c>
       <c r="I24" s="3">
-        <f>IF(AND($A24=""),"",IF(OR(($E24=""),($B24="")),"",(IF(ISNUMBER($E24),IF($E24=0,"0",ROUND($E24,9-INT(LOG10(ABS($E24))))&amp;""),$E24&amp;"")&amp;"|"&amp;IF(ISNUMBER($B24),IF($B24=0,"0",ROUND($B24,9-INT(LOG10(ABS($B24))))&amp;""),$B24&amp;""))))</f>
+        <f>IF(AND($A24=""),"",(IF(ISNUMBER($B24),IF($B24=0,"0",ROUND($B24,9-INT(LOG10(ABS($B24))))&amp;""),$B24&amp;"")&amp;" "&amp;IF(ISNUMBER($C24),IF($C24=0,"0",ROUND($C24,9-INT(LOG10(ABS($C24))))&amp;""),$C24&amp;"")&amp;" "&amp;IF(ISNUMBER($D24),IF($D24=0,"0",ROUND($D24,9-INT(LOG10(ABS($D24))))&amp;""),$D24&amp;"")))</f>
         <v/>
       </c>
       <c r="J24" s="3">
-        <f>IF(AND($A24=""),"",(IF(ISNUMBER($B24),IF($B24=0,"0",ROUND($B24,9-INT(LOG10(ABS($B24))))&amp;""),$B24&amp;"")&amp;" "&amp;IF(ISNUMBER($C24),IF($C24=0,"0",ROUND($C24,9-INT(LOG10(ABS($C24))))&amp;""),$C24&amp;"")&amp;" "&amp;IF(ISNUMBER($D24),IF($D24=0,"0",ROUND($D24,9-INT(LOG10(ABS($D24))))&amp;""),$D24&amp;"")))</f>
+        <f>IF(AND($A24=""),"",IF(OR(($E24=""),($B24="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E24))*(EXACT('Asignacion'!$B$4:$B$34,$B24)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E24))*(EXACT('Asignacion'!$B$4:$B$34,$B24)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E24))*(EXACT('Asignacion'!$B$4:$B$34,$B24)),0),0))))))</f>
         <v/>
       </c>
       <c r="K24" s="3">
-        <f>IF(AND($A24=""),"",IF(EXACT($I24,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I24)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I24)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I24)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A24=""),"",IF(AND(NOT(EXACT($J24,"")),EXACT($J24,$I24)),1,0))</f>
         <v/>
       </c>
       <c r="L24" s="3">
-        <f>IF(AND($A24=""),"",IF(AND(NOT(EXACT($I24,"")),EXACT($K24,$J24)),1,0))</f>
+        <f>IF(AND($A24=""),"",MID(IF(AND(NOT(($B24="")),($E24="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M24" s="3">
-        <f>IF(AND($A24=""),"",MID(IF(AND(NOT(($B24="")),($E24="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N24" s="3">
         <f>IF(OR(AND(NOT(($B24="")),($E24=""))),2,0)</f>
         <v/>
       </c>
@@ -1671,26 +1581,22 @@
         <v/>
       </c>
       <c r="I25" s="3">
-        <f>IF(AND($A25=""),"",IF(OR(($E25=""),($B25="")),"",(IF(ISNUMBER($E25),IF($E25=0,"0",ROUND($E25,9-INT(LOG10(ABS($E25))))&amp;""),$E25&amp;"")&amp;"|"&amp;IF(ISNUMBER($B25),IF($B25=0,"0",ROUND($B25,9-INT(LOG10(ABS($B25))))&amp;""),$B25&amp;""))))</f>
+        <f>IF(AND($A25=""),"",(IF(ISNUMBER($B25),IF($B25=0,"0",ROUND($B25,9-INT(LOG10(ABS($B25))))&amp;""),$B25&amp;"")&amp;" "&amp;IF(ISNUMBER($C25),IF($C25=0,"0",ROUND($C25,9-INT(LOG10(ABS($C25))))&amp;""),$C25&amp;"")&amp;" "&amp;IF(ISNUMBER($D25),IF($D25=0,"0",ROUND($D25,9-INT(LOG10(ABS($D25))))&amp;""),$D25&amp;"")))</f>
         <v/>
       </c>
       <c r="J25" s="3">
-        <f>IF(AND($A25=""),"",(IF(ISNUMBER($B25),IF($B25=0,"0",ROUND($B25,9-INT(LOG10(ABS($B25))))&amp;""),$B25&amp;"")&amp;" "&amp;IF(ISNUMBER($C25),IF($C25=0,"0",ROUND($C25,9-INT(LOG10(ABS($C25))))&amp;""),$C25&amp;"")&amp;" "&amp;IF(ISNUMBER($D25),IF($D25=0,"0",ROUND($D25,9-INT(LOG10(ABS($D25))))&amp;""),$D25&amp;"")))</f>
+        <f>IF(AND($A25=""),"",IF(OR(($E25=""),($B25="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E25))*(EXACT('Asignacion'!$B$4:$B$34,$B25)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E25))*(EXACT('Asignacion'!$B$4:$B$34,$B25)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E25))*(EXACT('Asignacion'!$B$4:$B$34,$B25)),0),0))))))</f>
         <v/>
       </c>
       <c r="K25" s="3">
-        <f>IF(AND($A25=""),"",IF(EXACT($I25,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I25)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I25)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I25)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A25=""),"",IF(AND(NOT(EXACT($J25,"")),EXACT($J25,$I25)),1,0))</f>
         <v/>
       </c>
       <c r="L25" s="3">
-        <f>IF(AND($A25=""),"",IF(AND(NOT(EXACT($I25,"")),EXACT($K25,$J25)),1,0))</f>
+        <f>IF(AND($A25=""),"",MID(IF(AND(NOT(($B25="")),($E25="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M25" s="3">
-        <f>IF(AND($A25=""),"",MID(IF(AND(NOT(($B25="")),($E25="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N25" s="3">
         <f>IF(OR(AND(NOT(($B25="")),($E25=""))),2,0)</f>
         <v/>
       </c>
@@ -1714,26 +1620,22 @@
         <v/>
       </c>
       <c r="I26" s="3">
-        <f>IF(AND($A26=""),"",IF(OR(($E26=""),($B26="")),"",(IF(ISNUMBER($E26),IF($E26=0,"0",ROUND($E26,9-INT(LOG10(ABS($E26))))&amp;""),$E26&amp;"")&amp;"|"&amp;IF(ISNUMBER($B26),IF($B26=0,"0",ROUND($B26,9-INT(LOG10(ABS($B26))))&amp;""),$B26&amp;""))))</f>
+        <f>IF(AND($A26=""),"",(IF(ISNUMBER($B26),IF($B26=0,"0",ROUND($B26,9-INT(LOG10(ABS($B26))))&amp;""),$B26&amp;"")&amp;" "&amp;IF(ISNUMBER($C26),IF($C26=0,"0",ROUND($C26,9-INT(LOG10(ABS($C26))))&amp;""),$C26&amp;"")&amp;" "&amp;IF(ISNUMBER($D26),IF($D26=0,"0",ROUND($D26,9-INT(LOG10(ABS($D26))))&amp;""),$D26&amp;"")))</f>
         <v/>
       </c>
       <c r="J26" s="3">
-        <f>IF(AND($A26=""),"",(IF(ISNUMBER($B26),IF($B26=0,"0",ROUND($B26,9-INT(LOG10(ABS($B26))))&amp;""),$B26&amp;"")&amp;" "&amp;IF(ISNUMBER($C26),IF($C26=0,"0",ROUND($C26,9-INT(LOG10(ABS($C26))))&amp;""),$C26&amp;"")&amp;" "&amp;IF(ISNUMBER($D26),IF($D26=0,"0",ROUND($D26,9-INT(LOG10(ABS($D26))))&amp;""),$D26&amp;"")))</f>
+        <f>IF(AND($A26=""),"",IF(OR(($E26=""),($B26="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E26))*(EXACT('Asignacion'!$B$4:$B$34,$B26)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E26))*(EXACT('Asignacion'!$B$4:$B$34,$B26)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E26))*(EXACT('Asignacion'!$B$4:$B$34,$B26)),0),0))))))</f>
         <v/>
       </c>
       <c r="K26" s="3">
-        <f>IF(AND($A26=""),"",IF(EXACT($I26,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I26)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I26)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I26)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A26=""),"",IF(AND(NOT(EXACT($J26,"")),EXACT($J26,$I26)),1,0))</f>
         <v/>
       </c>
       <c r="L26" s="3">
-        <f>IF(AND($A26=""),"",IF(AND(NOT(EXACT($I26,"")),EXACT($K26,$J26)),1,0))</f>
+        <f>IF(AND($A26=""),"",MID(IF(AND(NOT(($B26="")),($E26="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M26" s="3">
-        <f>IF(AND($A26=""),"",MID(IF(AND(NOT(($B26="")),($E26="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N26" s="3">
         <f>IF(OR(AND(NOT(($B26="")),($E26=""))),2,0)</f>
         <v/>
       </c>
@@ -1757,26 +1659,22 @@
         <v/>
       </c>
       <c r="I27" s="3">
-        <f>IF(AND($A27=""),"",IF(OR(($E27=""),($B27="")),"",(IF(ISNUMBER($E27),IF($E27=0,"0",ROUND($E27,9-INT(LOG10(ABS($E27))))&amp;""),$E27&amp;"")&amp;"|"&amp;IF(ISNUMBER($B27),IF($B27=0,"0",ROUND($B27,9-INT(LOG10(ABS($B27))))&amp;""),$B27&amp;""))))</f>
+        <f>IF(AND($A27=""),"",(IF(ISNUMBER($B27),IF($B27=0,"0",ROUND($B27,9-INT(LOG10(ABS($B27))))&amp;""),$B27&amp;"")&amp;" "&amp;IF(ISNUMBER($C27),IF($C27=0,"0",ROUND($C27,9-INT(LOG10(ABS($C27))))&amp;""),$C27&amp;"")&amp;" "&amp;IF(ISNUMBER($D27),IF($D27=0,"0",ROUND($D27,9-INT(LOG10(ABS($D27))))&amp;""),$D27&amp;"")))</f>
         <v/>
       </c>
       <c r="J27" s="3">
-        <f>IF(AND($A27=""),"",(IF(ISNUMBER($B27),IF($B27=0,"0",ROUND($B27,9-INT(LOG10(ABS($B27))))&amp;""),$B27&amp;"")&amp;" "&amp;IF(ISNUMBER($C27),IF($C27=0,"0",ROUND($C27,9-INT(LOG10(ABS($C27))))&amp;""),$C27&amp;"")&amp;" "&amp;IF(ISNUMBER($D27),IF($D27=0,"0",ROUND($D27,9-INT(LOG10(ABS($D27))))&amp;""),$D27&amp;"")))</f>
+        <f>IF(AND($A27=""),"",IF(OR(($E27=""),($B27="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E27))*(EXACT('Asignacion'!$B$4:$B$34,$B27)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E27))*(EXACT('Asignacion'!$B$4:$B$34,$B27)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E27))*(EXACT('Asignacion'!$B$4:$B$34,$B27)),0),0))))))</f>
         <v/>
       </c>
       <c r="K27" s="3">
-        <f>IF(AND($A27=""),"",IF(EXACT($I27,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I27)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I27)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I27)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A27=""),"",IF(AND(NOT(EXACT($J27,"")),EXACT($J27,$I27)),1,0))</f>
         <v/>
       </c>
       <c r="L27" s="3">
-        <f>IF(AND($A27=""),"",IF(AND(NOT(EXACT($I27,"")),EXACT($K27,$J27)),1,0))</f>
+        <f>IF(AND($A27=""),"",MID(IF(AND(NOT(($B27="")),($E27="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M27" s="3">
-        <f>IF(AND($A27=""),"",MID(IF(AND(NOT(($B27="")),($E27="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N27" s="3">
         <f>IF(OR(AND(NOT(($B27="")),($E27=""))),2,0)</f>
         <v/>
       </c>
@@ -1800,26 +1698,22 @@
         <v/>
       </c>
       <c r="I28" s="3">
-        <f>IF(AND($A28=""),"",IF(OR(($E28=""),($B28="")),"",(IF(ISNUMBER($E28),IF($E28=0,"0",ROUND($E28,9-INT(LOG10(ABS($E28))))&amp;""),$E28&amp;"")&amp;"|"&amp;IF(ISNUMBER($B28),IF($B28=0,"0",ROUND($B28,9-INT(LOG10(ABS($B28))))&amp;""),$B28&amp;""))))</f>
+        <f>IF(AND($A28=""),"",(IF(ISNUMBER($B28),IF($B28=0,"0",ROUND($B28,9-INT(LOG10(ABS($B28))))&amp;""),$B28&amp;"")&amp;" "&amp;IF(ISNUMBER($C28),IF($C28=0,"0",ROUND($C28,9-INT(LOG10(ABS($C28))))&amp;""),$C28&amp;"")&amp;" "&amp;IF(ISNUMBER($D28),IF($D28=0,"0",ROUND($D28,9-INT(LOG10(ABS($D28))))&amp;""),$D28&amp;"")))</f>
         <v/>
       </c>
       <c r="J28" s="3">
-        <f>IF(AND($A28=""),"",(IF(ISNUMBER($B28),IF($B28=0,"0",ROUND($B28,9-INT(LOG10(ABS($B28))))&amp;""),$B28&amp;"")&amp;" "&amp;IF(ISNUMBER($C28),IF($C28=0,"0",ROUND($C28,9-INT(LOG10(ABS($C28))))&amp;""),$C28&amp;"")&amp;" "&amp;IF(ISNUMBER($D28),IF($D28=0,"0",ROUND($D28,9-INT(LOG10(ABS($D28))))&amp;""),$D28&amp;"")))</f>
+        <f>IF(AND($A28=""),"",IF(OR(($E28=""),($B28="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E28))*(EXACT('Asignacion'!$B$4:$B$34,$B28)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E28))*(EXACT('Asignacion'!$B$4:$B$34,$B28)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E28))*(EXACT('Asignacion'!$B$4:$B$34,$B28)),0),0))))))</f>
         <v/>
       </c>
       <c r="K28" s="3">
-        <f>IF(AND($A28=""),"",IF(EXACT($I28,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I28)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I28)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I28)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A28=""),"",IF(AND(NOT(EXACT($J28,"")),EXACT($J28,$I28)),1,0))</f>
         <v/>
       </c>
       <c r="L28" s="3">
-        <f>IF(AND($A28=""),"",IF(AND(NOT(EXACT($I28,"")),EXACT($K28,$J28)),1,0))</f>
+        <f>IF(AND($A28=""),"",MID(IF(AND(NOT(($B28="")),($E28="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M28" s="3">
-        <f>IF(AND($A28=""),"",MID(IF(AND(NOT(($B28="")),($E28="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N28" s="3">
         <f>IF(OR(AND(NOT(($B28="")),($E28=""))),2,0)</f>
         <v/>
       </c>
@@ -1843,26 +1737,22 @@
         <v/>
       </c>
       <c r="I29" s="3">
-        <f>IF(AND($A29=""),"",IF(OR(($E29=""),($B29="")),"",(IF(ISNUMBER($E29),IF($E29=0,"0",ROUND($E29,9-INT(LOG10(ABS($E29))))&amp;""),$E29&amp;"")&amp;"|"&amp;IF(ISNUMBER($B29),IF($B29=0,"0",ROUND($B29,9-INT(LOG10(ABS($B29))))&amp;""),$B29&amp;""))))</f>
+        <f>IF(AND($A29=""),"",(IF(ISNUMBER($B29),IF($B29=0,"0",ROUND($B29,9-INT(LOG10(ABS($B29))))&amp;""),$B29&amp;"")&amp;" "&amp;IF(ISNUMBER($C29),IF($C29=0,"0",ROUND($C29,9-INT(LOG10(ABS($C29))))&amp;""),$C29&amp;"")&amp;" "&amp;IF(ISNUMBER($D29),IF($D29=0,"0",ROUND($D29,9-INT(LOG10(ABS($D29))))&amp;""),$D29&amp;"")))</f>
         <v/>
       </c>
       <c r="J29" s="3">
-        <f>IF(AND($A29=""),"",(IF(ISNUMBER($B29),IF($B29=0,"0",ROUND($B29,9-INT(LOG10(ABS($B29))))&amp;""),$B29&amp;"")&amp;" "&amp;IF(ISNUMBER($C29),IF($C29=0,"0",ROUND($C29,9-INT(LOG10(ABS($C29))))&amp;""),$C29&amp;"")&amp;" "&amp;IF(ISNUMBER($D29),IF($D29=0,"0",ROUND($D29,9-INT(LOG10(ABS($D29))))&amp;""),$D29&amp;"")))</f>
+        <f>IF(AND($A29=""),"",IF(OR(($E29=""),($B29="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E29))*(EXACT('Asignacion'!$B$4:$B$34,$B29)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E29))*(EXACT('Asignacion'!$B$4:$B$34,$B29)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E29))*(EXACT('Asignacion'!$B$4:$B$34,$B29)),0),0))))))</f>
         <v/>
       </c>
       <c r="K29" s="3">
-        <f>IF(AND($A29=""),"",IF(EXACT($I29,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I29)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I29)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I29)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A29=""),"",IF(AND(NOT(EXACT($J29,"")),EXACT($J29,$I29)),1,0))</f>
         <v/>
       </c>
       <c r="L29" s="3">
-        <f>IF(AND($A29=""),"",IF(AND(NOT(EXACT($I29,"")),EXACT($K29,$J29)),1,0))</f>
+        <f>IF(AND($A29=""),"",MID(IF(AND(NOT(($B29="")),($E29="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M29" s="3">
-        <f>IF(AND($A29=""),"",MID(IF(AND(NOT(($B29="")),($E29="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N29" s="3">
         <f>IF(OR(AND(NOT(($B29="")),($E29=""))),2,0)</f>
         <v/>
       </c>
@@ -1886,26 +1776,22 @@
         <v/>
       </c>
       <c r="I30" s="3">
-        <f>IF(AND($A30=""),"",IF(OR(($E30=""),($B30="")),"",(IF(ISNUMBER($E30),IF($E30=0,"0",ROUND($E30,9-INT(LOG10(ABS($E30))))&amp;""),$E30&amp;"")&amp;"|"&amp;IF(ISNUMBER($B30),IF($B30=0,"0",ROUND($B30,9-INT(LOG10(ABS($B30))))&amp;""),$B30&amp;""))))</f>
+        <f>IF(AND($A30=""),"",(IF(ISNUMBER($B30),IF($B30=0,"0",ROUND($B30,9-INT(LOG10(ABS($B30))))&amp;""),$B30&amp;"")&amp;" "&amp;IF(ISNUMBER($C30),IF($C30=0,"0",ROUND($C30,9-INT(LOG10(ABS($C30))))&amp;""),$C30&amp;"")&amp;" "&amp;IF(ISNUMBER($D30),IF($D30=0,"0",ROUND($D30,9-INT(LOG10(ABS($D30))))&amp;""),$D30&amp;"")))</f>
         <v/>
       </c>
       <c r="J30" s="3">
-        <f>IF(AND($A30=""),"",(IF(ISNUMBER($B30),IF($B30=0,"0",ROUND($B30,9-INT(LOG10(ABS($B30))))&amp;""),$B30&amp;"")&amp;" "&amp;IF(ISNUMBER($C30),IF($C30=0,"0",ROUND($C30,9-INT(LOG10(ABS($C30))))&amp;""),$C30&amp;"")&amp;" "&amp;IF(ISNUMBER($D30),IF($D30=0,"0",ROUND($D30,9-INT(LOG10(ABS($D30))))&amp;""),$D30&amp;"")))</f>
+        <f>IF(AND($A30=""),"",IF(OR(($E30=""),($B30="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E30))*(EXACT('Asignacion'!$B$4:$B$34,$B30)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E30))*(EXACT('Asignacion'!$B$4:$B$34,$B30)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E30))*(EXACT('Asignacion'!$B$4:$B$34,$B30)),0),0))))))</f>
         <v/>
       </c>
       <c r="K30" s="3">
-        <f>IF(AND($A30=""),"",IF(EXACT($I30,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I30)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I30)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I30)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A30=""),"",IF(AND(NOT(EXACT($J30,"")),EXACT($J30,$I30)),1,0))</f>
         <v/>
       </c>
       <c r="L30" s="3">
-        <f>IF(AND($A30=""),"",IF(AND(NOT(EXACT($I30,"")),EXACT($K30,$J30)),1,0))</f>
+        <f>IF(AND($A30=""),"",MID(IF(AND(NOT(($B30="")),($E30="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M30" s="3">
-        <f>IF(AND($A30=""),"",MID(IF(AND(NOT(($B30="")),($E30="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N30" s="3">
         <f>IF(OR(AND(NOT(($B30="")),($E30=""))),2,0)</f>
         <v/>
       </c>
@@ -1929,26 +1815,22 @@
         <v/>
       </c>
       <c r="I31" s="3">
-        <f>IF(AND($A31=""),"",IF(OR(($E31=""),($B31="")),"",(IF(ISNUMBER($E31),IF($E31=0,"0",ROUND($E31,9-INT(LOG10(ABS($E31))))&amp;""),$E31&amp;"")&amp;"|"&amp;IF(ISNUMBER($B31),IF($B31=0,"0",ROUND($B31,9-INT(LOG10(ABS($B31))))&amp;""),$B31&amp;""))))</f>
+        <f>IF(AND($A31=""),"",(IF(ISNUMBER($B31),IF($B31=0,"0",ROUND($B31,9-INT(LOG10(ABS($B31))))&amp;""),$B31&amp;"")&amp;" "&amp;IF(ISNUMBER($C31),IF($C31=0,"0",ROUND($C31,9-INT(LOG10(ABS($C31))))&amp;""),$C31&amp;"")&amp;" "&amp;IF(ISNUMBER($D31),IF($D31=0,"0",ROUND($D31,9-INT(LOG10(ABS($D31))))&amp;""),$D31&amp;"")))</f>
         <v/>
       </c>
       <c r="J31" s="3">
-        <f>IF(AND($A31=""),"",(IF(ISNUMBER($B31),IF($B31=0,"0",ROUND($B31,9-INT(LOG10(ABS($B31))))&amp;""),$B31&amp;"")&amp;" "&amp;IF(ISNUMBER($C31),IF($C31=0,"0",ROUND($C31,9-INT(LOG10(ABS($C31))))&amp;""),$C31&amp;"")&amp;" "&amp;IF(ISNUMBER($D31),IF($D31=0,"0",ROUND($D31,9-INT(LOG10(ABS($D31))))&amp;""),$D31&amp;"")))</f>
+        <f>IF(AND($A31=""),"",IF(OR(($E31=""),($B31="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E31))*(EXACT('Asignacion'!$B$4:$B$34,$B31)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E31))*(EXACT('Asignacion'!$B$4:$B$34,$B31)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E31))*(EXACT('Asignacion'!$B$4:$B$34,$B31)),0),0))))))</f>
         <v/>
       </c>
       <c r="K31" s="3">
-        <f>IF(AND($A31=""),"",IF(EXACT($I31,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I31)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I31)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I31)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A31=""),"",IF(AND(NOT(EXACT($J31,"")),EXACT($J31,$I31)),1,0))</f>
         <v/>
       </c>
       <c r="L31" s="3">
-        <f>IF(AND($A31=""),"",IF(AND(NOT(EXACT($I31,"")),EXACT($K31,$J31)),1,0))</f>
+        <f>IF(AND($A31=""),"",MID(IF(AND(NOT(($B31="")),($E31="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M31" s="3">
-        <f>IF(AND($A31=""),"",MID(IF(AND(NOT(($B31="")),($E31="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N31" s="3">
         <f>IF(OR(AND(NOT(($B31="")),($E31=""))),2,0)</f>
         <v/>
       </c>
@@ -1972,26 +1854,22 @@
         <v/>
       </c>
       <c r="I32" s="3">
-        <f>IF(AND($A32=""),"",IF(OR(($E32=""),($B32="")),"",(IF(ISNUMBER($E32),IF($E32=0,"0",ROUND($E32,9-INT(LOG10(ABS($E32))))&amp;""),$E32&amp;"")&amp;"|"&amp;IF(ISNUMBER($B32),IF($B32=0,"0",ROUND($B32,9-INT(LOG10(ABS($B32))))&amp;""),$B32&amp;""))))</f>
+        <f>IF(AND($A32=""),"",(IF(ISNUMBER($B32),IF($B32=0,"0",ROUND($B32,9-INT(LOG10(ABS($B32))))&amp;""),$B32&amp;"")&amp;" "&amp;IF(ISNUMBER($C32),IF($C32=0,"0",ROUND($C32,9-INT(LOG10(ABS($C32))))&amp;""),$C32&amp;"")&amp;" "&amp;IF(ISNUMBER($D32),IF($D32=0,"0",ROUND($D32,9-INT(LOG10(ABS($D32))))&amp;""),$D32&amp;"")))</f>
         <v/>
       </c>
       <c r="J32" s="3">
-        <f>IF(AND($A32=""),"",(IF(ISNUMBER($B32),IF($B32=0,"0",ROUND($B32,9-INT(LOG10(ABS($B32))))&amp;""),$B32&amp;"")&amp;" "&amp;IF(ISNUMBER($C32),IF($C32=0,"0",ROUND($C32,9-INT(LOG10(ABS($C32))))&amp;""),$C32&amp;"")&amp;" "&amp;IF(ISNUMBER($D32),IF($D32=0,"0",ROUND($D32,9-INT(LOG10(ABS($D32))))&amp;""),$D32&amp;"")))</f>
+        <f>IF(AND($A32=""),"",IF(OR(($E32=""),($B32="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E32))*(EXACT('Asignacion'!$B$4:$B$34,$B32)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E32))*(EXACT('Asignacion'!$B$4:$B$34,$B32)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E32))*(EXACT('Asignacion'!$B$4:$B$34,$B32)),0),0))))))</f>
         <v/>
       </c>
       <c r="K32" s="3">
-        <f>IF(AND($A32=""),"",IF(EXACT($I32,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I32)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I32)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I32)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A32=""),"",IF(AND(NOT(EXACT($J32,"")),EXACT($J32,$I32)),1,0))</f>
         <v/>
       </c>
       <c r="L32" s="3">
-        <f>IF(AND($A32=""),"",IF(AND(NOT(EXACT($I32,"")),EXACT($K32,$J32)),1,0))</f>
+        <f>IF(AND($A32=""),"",MID(IF(AND(NOT(($B32="")),($E32="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M32" s="3">
-        <f>IF(AND($A32=""),"",MID(IF(AND(NOT(($B32="")),($E32="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N32" s="3">
         <f>IF(OR(AND(NOT(($B32="")),($E32=""))),2,0)</f>
         <v/>
       </c>
@@ -2015,26 +1893,22 @@
         <v/>
       </c>
       <c r="I33" s="3">
-        <f>IF(AND($A33=""),"",IF(OR(($E33=""),($B33="")),"",(IF(ISNUMBER($E33),IF($E33=0,"0",ROUND($E33,9-INT(LOG10(ABS($E33))))&amp;""),$E33&amp;"")&amp;"|"&amp;IF(ISNUMBER($B33),IF($B33=0,"0",ROUND($B33,9-INT(LOG10(ABS($B33))))&amp;""),$B33&amp;""))))</f>
+        <f>IF(AND($A33=""),"",(IF(ISNUMBER($B33),IF($B33=0,"0",ROUND($B33,9-INT(LOG10(ABS($B33))))&amp;""),$B33&amp;"")&amp;" "&amp;IF(ISNUMBER($C33),IF($C33=0,"0",ROUND($C33,9-INT(LOG10(ABS($C33))))&amp;""),$C33&amp;"")&amp;" "&amp;IF(ISNUMBER($D33),IF($D33=0,"0",ROUND($D33,9-INT(LOG10(ABS($D33))))&amp;""),$D33&amp;"")))</f>
         <v/>
       </c>
       <c r="J33" s="3">
-        <f>IF(AND($A33=""),"",(IF(ISNUMBER($B33),IF($B33=0,"0",ROUND($B33,9-INT(LOG10(ABS($B33))))&amp;""),$B33&amp;"")&amp;" "&amp;IF(ISNUMBER($C33),IF($C33=0,"0",ROUND($C33,9-INT(LOG10(ABS($C33))))&amp;""),$C33&amp;"")&amp;" "&amp;IF(ISNUMBER($D33),IF($D33=0,"0",ROUND($D33,9-INT(LOG10(ABS($D33))))&amp;""),$D33&amp;"")))</f>
+        <f>IF(AND($A33=""),"",IF(OR(($E33=""),($B33="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E33))*(EXACT('Asignacion'!$B$4:$B$34,$B33)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E33))*(EXACT('Asignacion'!$B$4:$B$34,$B33)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E33))*(EXACT('Asignacion'!$B$4:$B$34,$B33)),0),0))))))</f>
         <v/>
       </c>
       <c r="K33" s="3">
-        <f>IF(AND($A33=""),"",IF(EXACT($I33,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I33)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I33)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I33)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A33=""),"",IF(AND(NOT(EXACT($J33,"")),EXACT($J33,$I33)),1,0))</f>
         <v/>
       </c>
       <c r="L33" s="3">
-        <f>IF(AND($A33=""),"",IF(AND(NOT(EXACT($I33,"")),EXACT($K33,$J33)),1,0))</f>
+        <f>IF(AND($A33=""),"",MID(IF(AND(NOT(($B33="")),($E33="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M33" s="3">
-        <f>IF(AND($A33=""),"",MID(IF(AND(NOT(($B33="")),($E33="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N33" s="3">
         <f>IF(OR(AND(NOT(($B33="")),($E33=""))),2,0)</f>
         <v/>
       </c>
@@ -2058,26 +1932,22 @@
         <v/>
       </c>
       <c r="I34" s="3">
-        <f>IF(AND($A34=""),"",IF(OR(($E34=""),($B34="")),"",(IF(ISNUMBER($E34),IF($E34=0,"0",ROUND($E34,9-INT(LOG10(ABS($E34))))&amp;""),$E34&amp;"")&amp;"|"&amp;IF(ISNUMBER($B34),IF($B34=0,"0",ROUND($B34,9-INT(LOG10(ABS($B34))))&amp;""),$B34&amp;""))))</f>
+        <f>IF(AND($A34=""),"",(IF(ISNUMBER($B34),IF($B34=0,"0",ROUND($B34,9-INT(LOG10(ABS($B34))))&amp;""),$B34&amp;"")&amp;" "&amp;IF(ISNUMBER($C34),IF($C34=0,"0",ROUND($C34,9-INT(LOG10(ABS($C34))))&amp;""),$C34&amp;"")&amp;" "&amp;IF(ISNUMBER($D34),IF($D34=0,"0",ROUND($D34,9-INT(LOG10(ABS($D34))))&amp;""),$D34&amp;"")))</f>
         <v/>
       </c>
       <c r="J34" s="3">
-        <f>IF(AND($A34=""),"",(IF(ISNUMBER($B34),IF($B34=0,"0",ROUND($B34,9-INT(LOG10(ABS($B34))))&amp;""),$B34&amp;"")&amp;" "&amp;IF(ISNUMBER($C34),IF($C34=0,"0",ROUND($C34,9-INT(LOG10(ABS($C34))))&amp;""),$C34&amp;"")&amp;" "&amp;IF(ISNUMBER($D34),IF($D34=0,"0",ROUND($D34,9-INT(LOG10(ABS($D34))))&amp;""),$D34&amp;"")))</f>
+        <f>IF(AND($A34=""),"",IF(OR(($E34=""),($B34="")),"",IF(ISNA(MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E34))*(EXACT('Asignacion'!$B$4:$B$34,$B34)),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E34))*(EXACT('Asignacion'!$B$4:$B$34,$B34)),0),0))),"",INDEX('Asignacion'!$I$4:$I$34,MATCH(1,INDEX(1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0)*(EXACT('Asignacion'!$E$4:$E$34,$E34))*(EXACT('Asignacion'!$B$4:$B$34,$B34)),0),0))))))</f>
         <v/>
       </c>
       <c r="K34" s="3">
-        <f>IF(AND($A34=""),"",IF(EXACT($I34,""),"",IF(ISNA(MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I34)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0)),"",IF(ISBLANK(INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I34)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))),"",INDEX('Asignacion'!$J$4:$J$34,MATCH(1,INDEX(EXACT('Asignacion'!$I$4:$I$34,$I34)*1*((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0),0),0))))))</f>
+        <f>IF(AND($A34=""),"",IF(AND(NOT(EXACT($J34,"")),EXACT($J34,$I34)),1,0))</f>
         <v/>
       </c>
       <c r="L34" s="3">
-        <f>IF(AND($A34=""),"",IF(AND(NOT(EXACT($I34,"")),EXACT($K34,$J34)),1,0))</f>
+        <f>IF(AND($A34=""),"",MID(IF(AND(NOT(($B34="")),($E34="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
         <v/>
       </c>
       <c r="M34" s="3">
-        <f>IF(AND($A34=""),"",MID(IF(AND(NOT(($B34="")),($E34="")),"; "&amp;"Esta fila de carga todavia no tiene profesor",""),3,32767))</f>
-        <v/>
-      </c>
-      <c r="N34" s="3">
         <f>IF(OR(AND(NOT(($B34="")),($E34=""))),2,0)</f>
         <v/>
       </c>
@@ -2219,7 +2089,7 @@
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>IF(AND($A4=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A4)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A4=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A4)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -2259,7 +2129,7 @@
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>IF(AND($A5=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A5)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A5=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A5)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -2299,7 +2169,7 @@
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>IF(AND($A6=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A6)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A6=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A6)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -2339,7 +2209,7 @@
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>IF(AND($A7=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A7)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A7=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A7)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -2365,7 +2235,7 @@
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>IF(AND($A8=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A8)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A8=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A8)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -2391,7 +2261,7 @@
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>IF(AND($A9=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A9)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A9=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A9)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -2417,7 +2287,7 @@
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>IF(AND($A10=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A10)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A10=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A10)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -2443,7 +2313,7 @@
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>IF(AND($A11=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A11)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A11=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A11)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -2469,7 +2339,7 @@
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>IF(AND($A12=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A12)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A12=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A12)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -2495,7 +2365,7 @@
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>IF(AND($A13=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A13)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A13=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A13)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -2521,7 +2391,7 @@
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>IF(AND($A14=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A14)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A14=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A14)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G14" s="3">
@@ -2547,7 +2417,7 @@
         <v/>
       </c>
       <c r="F15" s="3">
-        <f>IF(AND($A15=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A15)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A15=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A15)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G15" s="3">
@@ -2573,7 +2443,7 @@
         <v/>
       </c>
       <c r="F16" s="3">
-        <f>IF(AND($A16=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A16)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A16=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A16)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G16" s="3">
@@ -2599,7 +2469,7 @@
         <v/>
       </c>
       <c r="F17" s="3">
-        <f>IF(AND($A17=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A17)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A17=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A17)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G17" s="3">
@@ -2625,7 +2495,7 @@
         <v/>
       </c>
       <c r="F18" s="3">
-        <f>IF(AND($A18=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A18)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A18=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A18)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G18" s="3">
@@ -2651,7 +2521,7 @@
         <v/>
       </c>
       <c r="F19" s="3">
-        <f>IF(AND($A19=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A19)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A19=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A19)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G19" s="3">
@@ -2677,7 +2547,7 @@
         <v/>
       </c>
       <c r="F20" s="3">
-        <f>IF(AND($A20=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A20)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A20=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A20)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G20" s="3">
@@ -2703,7 +2573,7 @@
         <v/>
       </c>
       <c r="F21" s="3">
-        <f>IF(AND($A21=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A21)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A21=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A21)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G21" s="3">
@@ -2729,7 +2599,7 @@
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>IF(AND($A22=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A22)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A22=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A22)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G22" s="3">
@@ -2755,7 +2625,7 @@
         <v/>
       </c>
       <c r="F23" s="3">
-        <f>IF(AND($A23=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A23)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A23=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A23)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G23" s="3">
@@ -2781,7 +2651,7 @@
         <v/>
       </c>
       <c r="F24" s="3">
-        <f>IF(AND($A24=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A24)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A24=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A24)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G24" s="3">
@@ -2807,7 +2677,7 @@
         <v/>
       </c>
       <c r="F25" s="3">
-        <f>IF(AND($A25=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A25)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A25=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A25)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G25" s="3">
@@ -2833,7 +2703,7 @@
         <v/>
       </c>
       <c r="F26" s="3">
-        <f>IF(AND($A26=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A26)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A26=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A26)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G26" s="3">
@@ -2859,7 +2729,7 @@
         <v/>
       </c>
       <c r="F27" s="3">
-        <f>IF(AND($A27=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A27)))*(IFERROR(VALUE('Asignacion'!$L$4:$L$34&amp;""),0))))</f>
+        <f>IF(AND($A27=""),"",SUMPRODUCT(1*(((('Asignacion'!$A$4:$A$34&lt;&gt;""))&gt;0))*((EXACT('Asignacion'!$E$4:$E$34,$A27)))*(IFERROR(VALUE('Asignacion'!$K$4:$K$34&amp;""),0))))</f>
         <v/>
       </c>
       <c r="G27" s="3">
@@ -4097,7 +3967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A1:X27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4109,9 +3979,9 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
@@ -4122,9 +3992,7 @@
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4182,81 +4050,71 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Par</t>
+          <t>Codigo</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
+          <t>Primera del par</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Profesor</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Asignatura</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
           <t>Codigo</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>Primera del par</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>Profesor</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>Asignatura</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>Horas</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>Par</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>Codigo</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>Primera del par</t>
-        </is>
-      </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="X3" s="9" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
@@ -4301,7 +4159,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>PIAD|EST-CC</t>
+          <t xml:space="preserve">EST-CC Conf </t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -4309,20 +4167,16 @@
           <t xml:space="preserve">EST-CC Conf </t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EST-CC Conf </t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="n">
+      <c r="L4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>PIAD</t>
         </is>
       </c>
+      <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="n"/>
@@ -4331,8 +4185,6 @@
       <c r="U4" s="3" t="n"/>
       <c r="V4" s="3" t="n"/>
       <c r="W4" s="3" t="n"/>
-      <c r="X4" s="3" t="n"/>
-      <c r="Y4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3">
@@ -4377,69 +4229,60 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>PIAD|EST-CC</t>
+          <t>EST-CC CP 1</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>EST-CC CP 1</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
           <t xml:space="preserve">EST-CC Conf </t>
         </is>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X5" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y5" s="3">
+      <c r="X5">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z5">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -4486,69 +4329,60 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>PIAD|EST-CC</t>
+          <t>EST-CC CP 2</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>EST-CC CP 2</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
           <t xml:space="preserve">EST-CC Conf </t>
         </is>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="L6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X6" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y6" s="3">
+      <c r="X6">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z6">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -4591,7 +4425,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>PIAD|EST-MAT</t>
+          <t xml:space="preserve">EST-MAT Conf </t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -4599,61 +4433,52 @@
           <t xml:space="preserve">EST-MAT Conf </t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EST-MAT Conf </t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="n">
+      <c r="L7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W7" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X7" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y7" s="3">
+      <c r="X7">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z7">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -4696,7 +4521,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>MARA|PROB</t>
+          <t xml:space="preserve">PROB Conf </t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -4704,61 +4529,52 @@
           <t xml:space="preserve">PROB Conf </t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROB Conf </t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="n">
+      <c r="L8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W8" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X8" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y8" s="3">
+      <c r="X8">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z8">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -4805,69 +4621,60 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>MARA|PROB</t>
+          <t>PROB CP 1</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>PROB CP 1</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
           <t xml:space="preserve">PROB Conf </t>
         </is>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="L9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
+      <c r="N9" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W9" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X9" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y9" s="3">
+      <c r="X9">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z9">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"PIAD"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -4910,7 +4717,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>MARA|MNUM</t>
+          <t xml:space="preserve">MNUM Conf </t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -4918,20 +4725,16 @@
           <t xml:space="preserve">MNUM Conf </t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MNUM Conf </t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="n">
+      <c r="L10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>MARA</t>
         </is>
       </c>
+      <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
       <c r="Q10" s="3" t="n"/>
       <c r="R10" s="3" t="n"/>
@@ -4940,8 +4743,6 @@
       <c r="U10" s="3" t="n"/>
       <c r="V10" s="3" t="n"/>
       <c r="W10" s="3" t="n"/>
-      <c r="X10" s="3" t="n"/>
-      <c r="Y10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3">
@@ -4986,7 +4787,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>LUGO|EST-MAT</t>
+          <t>EST-MAT CP 1</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4994,61 +4795,52 @@
           <t>EST-MAT CP 1</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>EST-MAT CP 1</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="n">
+      <c r="L11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
+      <c r="N11" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W11" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X11" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y11" s="3">
+      <c r="X11">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z11">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5066,53 +4858,48 @@
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
+      <c r="N12" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W12" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X12" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y12" s="3">
+      <c r="X12">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z12">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5130,53 +4917,48 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
+      <c r="N13" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W13" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X13" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y13" s="3">
+      <c r="X13">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z13">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5194,53 +4976,48 @@
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W14" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X14" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y14" s="3">
+      <c r="X14">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z14">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5258,53 +5035,48 @@
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
+      <c r="N15" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W15" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X15" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y15" s="3">
+      <c r="X15">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z15">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"MARA"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5322,12 +5094,12 @@
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>LUGO</t>
         </is>
       </c>
+      <c r="O16" s="3" t="n"/>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="n"/>
       <c r="R16" s="3" t="n"/>
@@ -5336,8 +5108,6 @@
       <c r="U16" s="3" t="n"/>
       <c r="V16" s="3" t="n"/>
       <c r="W16" s="3" t="n"/>
-      <c r="X16" s="3" t="n"/>
-      <c r="Y16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -5353,53 +5123,48 @@
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
+      <c r="N17" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W17" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X17" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y17" s="3">
+      <c r="X17">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z17">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5417,53 +5182,48 @@
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
+      <c r="N18" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W18" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X18" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y18" s="3">
+      <c r="X18">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z18">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5481,53 +5241,48 @@
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
+      <c r="N19" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W19" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X19" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y19" s="3">
+      <c r="X19">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z19">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5545,53 +5300,48 @@
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
+      <c r="N20" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W20" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X20" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y20" s="3">
+      <c r="X20">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z20">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5609,53 +5359,48 @@
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
+      <c r="N21" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W21" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X21" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y21" s="3">
+      <c r="X21">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z21">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"LUGO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5673,12 +5418,12 @@
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>ROTO</t>
         </is>
       </c>
+      <c r="O22" s="3" t="n"/>
       <c r="P22" s="3" t="n"/>
       <c r="Q22" s="3" t="n"/>
       <c r="R22" s="3" t="n"/>
@@ -5687,8 +5432,6 @@
       <c r="U22" s="3" t="n"/>
       <c r="V22" s="3" t="n"/>
       <c r="W22" s="3" t="n"/>
-      <c r="X22" s="3" t="n"/>
-      <c r="Y22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -5704,53 +5447,48 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="n"/>
       <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
+      <c r="N23" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W23" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X23" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y23" s="3">
+      <c r="X23">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z23">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"1")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5768,53 +5506,48 @@
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
+      <c r="N24" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W24" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X24" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y24" s="3">
+      <c r="X24">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z24">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"2")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5832,53 +5565,48 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
+      <c r="N25" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W25" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X25" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y25" s="3">
+      <c r="X25">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z25">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"3")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5896,53 +5624,48 @@
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
       <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
+      <c r="N26" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W26" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X26" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y26" s="3">
+      <c r="X26">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z26">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"4")*1,0),0))))</f>
         <v/>
       </c>
     </row>
@@ -5960,53 +5683,48 @@
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
+      <c r="N27" s="3">
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <v/>
+      </c>
       <c r="O27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$B$4:$B$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="P27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$C$4:$C$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="Q27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$D$4:$D$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="R27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$E$4:$E$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="S27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$F$4:$F$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="T27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$G$4:$G$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="U27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$H$4:$H$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="V27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$I$4:$I$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
+        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
       <c r="W27" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$J$4:$J$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="X27" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$K$4:$K$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
-      <c r="Y27" s="3">
+      <c r="X27">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$L$4:$L$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="Z27">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0)),"",IF(ISBLANK(INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))),"",INDEX('Detalle - Lo que imparte'!$M$4:$M$11,MATCH(1,INDEX(EXACT('Detalle - Lo que imparte'!$A$4:$A$11,"ROTO"&amp;CHAR(30)&amp;"5")*1,0),0))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the example outputs with legend sentences and editable parameters
</commit_message>
<xml_diff>
--- a/ejemplos/resultados/departamento.xlsx
+++ b/ejemplos/resultados/departamento.xlsx
@@ -2756,7 +2756,7 @@
       <c r="A30" s="7" t="n"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>sobrecarga</t>
+          <t>El profesor pasa de su tope de horas</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
       <c r="A30" s="6" t="n"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>cobertura incompleta</t>
+          <t>La asignatura no tiene cubiertas todas sus horas</t>
         </is>
       </c>
     </row>
@@ -3933,7 +3933,7 @@
       <c r="A31" s="8" t="n"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>cobertura completa</t>
+          <t>La asignatura tiene cubiertas todas sus horas</t>
         </is>
       </c>
     </row>

</xml_diff>